<commit_message>
panel 1: replace Yi Tian Thung with Dr Maggie Sou (photo, bio, programme, xlsx)
</commit_message>
<xml_diff>
--- a/public/events/Program.xlsx
+++ b/public/events/Program.xlsx
@@ -313,9 +313,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -664,14 +662,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C4" s="20" t="inlineStr">
+      <c r="C4" s="58" t="inlineStr">
         <is>
           <t>Breakfast &amp; Registration</t>
         </is>
       </c>
-      <c r="D4" s="20" t="n"/>
-      <c r="E4" s="20" t="n"/>
-      <c r="F4" s="20" t="n"/>
+      <c r="D4" s="58" t="n"/>
+      <c r="E4" s="58" t="n"/>
+      <c r="F4" s="58" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="17" t="inlineStr">
@@ -684,18 +682,18 @@
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="C5" s="58" t="inlineStr">
         <is>
           <t>Opening Ceremony</t>
         </is>
       </c>
-      <c r="D5" s="20" t="n"/>
-      <c r="E5" s="20" t="inlineStr">
+      <c r="D5" s="58" t="n"/>
+      <c r="E5" s="58" t="inlineStr">
         <is>
           <t>Mdm Rahayu Mahzam</t>
         </is>
       </c>
-      <c r="F5" s="20" t="inlineStr">
+      <c r="F5" s="58" t="inlineStr">
         <is>
           <t>Guest-of-Honour; Opening Address</t>
         </is>
@@ -712,18 +710,18 @@
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C6" s="20" t="inlineStr">
+      <c r="C6" s="58" t="inlineStr">
         <is>
           <t>Opening Ceremony</t>
         </is>
       </c>
-      <c r="D6" s="20" t="n"/>
-      <c r="E6" s="20" t="inlineStr">
+      <c r="D6" s="58" t="n"/>
+      <c r="E6" s="58" t="inlineStr">
         <is>
           <t>H.E. Alexandra Baumann</t>
         </is>
       </c>
-      <c r="F6" s="20" t="inlineStr">
+      <c r="F6" s="58" t="inlineStr">
         <is>
           <t>VVIP; Ambassador of Switzerland to Singapore</t>
         </is>
@@ -740,18 +738,18 @@
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C7" s="20" t="inlineStr">
+      <c r="C7" s="58" t="inlineStr">
         <is>
           <t>Opening Ceremony</t>
         </is>
       </c>
-      <c r="D7" s="20" t="n"/>
-      <c r="E7" s="20" t="inlineStr">
+      <c r="D7" s="58" t="n"/>
+      <c r="E7" s="58" t="inlineStr">
         <is>
           <t>Eduard Ruge</t>
         </is>
       </c>
-      <c r="F7" s="20" t="inlineStr">
+      <c r="F7" s="58" t="inlineStr">
         <is>
           <t>VVIP;  Counsellor of German Embassy for Cooperation in Science, Technology and Research</t>
         </is>
@@ -768,18 +766,18 @@
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C8" s="20" t="inlineStr">
+      <c r="C8" s="58" t="inlineStr">
         <is>
           <t>AI Algo Trading Hackathon Award Ceremony</t>
         </is>
       </c>
-      <c r="D8" s="20" t="n"/>
-      <c r="E8" s="20" t="inlineStr">
+      <c r="D8" s="58" t="n"/>
+      <c r="E8" s="58" t="inlineStr">
         <is>
           <t>Mdm Rahayu Mahzam; H.E. Alexandra Baumann</t>
         </is>
       </c>
-      <c r="F8" s="20" t="inlineStr">
+      <c r="F8" s="58" t="inlineStr">
         <is>
           <t>Award presenters</t>
         </is>
@@ -796,18 +794,18 @@
           <t>Outside</t>
         </is>
       </c>
-      <c r="C9" s="20" t="inlineStr">
+      <c r="C9" s="58" t="inlineStr">
         <is>
           <t>Official Group Photograph</t>
         </is>
       </c>
-      <c r="D9" s="20" t="n"/>
-      <c r="E9" s="20" t="inlineStr">
+      <c r="D9" s="58" t="n"/>
+      <c r="E9" s="58" t="inlineStr">
         <is>
           <t>Guest-of-Honour, VIPs &amp; all participants</t>
         </is>
       </c>
-      <c r="F9" s="20" t="inlineStr">
+      <c r="F9" s="58" t="inlineStr">
         <is>
           <t>Group photograph</t>
         </is>
@@ -824,22 +822,22 @@
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="51" t="inlineStr">
         <is>
           <t>Keynote 1</t>
         </is>
       </c>
-      <c r="D10" s="18" t="inlineStr">
+      <c r="D10" s="52" t="inlineStr">
         <is>
           <t>Chair: Ying Chen</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="51" t="inlineStr">
         <is>
           <t>Stefan Woerner, IBM Research Switzerland</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="51" t="inlineStr">
         <is>
           <t>Towards Practical Quantum Advantage</t>
         </is>
@@ -876,18 +874,18 @@
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C11" s="24" t="inlineStr">
+      <c r="C11" s="40" t="inlineStr">
         <is>
           <t>Showcase 1</t>
         </is>
       </c>
-      <c r="D11" s="24" t="n"/>
-      <c r="E11" s="24" t="inlineStr">
+      <c r="D11" s="40" t="n"/>
+      <c r="E11" s="40" t="inlineStr">
         <is>
           <t>Jeremy Woo, Senior Technical Advisor, D-Wave</t>
         </is>
       </c>
-      <c r="F11" s="24" t="inlineStr">
+      <c r="F11" s="40" t="inlineStr">
         <is>
           <t>Annealing and Dual-Rail Cavity Qubit Quantum Computers: How Do Advances in Annealing and Gate-Model Quantum Computers Affect Industry?</t>
         </is>
@@ -924,22 +922,22 @@
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C12" s="37" t="inlineStr">
+      <c r="C12" s="44" t="inlineStr">
         <is>
           <t>Panel 1: Agentic AI and Autonomous Systems</t>
         </is>
       </c>
-      <c r="D12" s="37" t="inlineStr">
+      <c r="D12" s="44" t="inlineStr">
         <is>
           <t>Moderator: Thorsten Koch</t>
         </is>
       </c>
-      <c r="E12" s="37" t="inlineStr">
-        <is>
-          <t>Si Min Chan, NVIDIA; Masahiro Horibe, AIST G-QuAT; Yi Tian Thung, Singapore Maritime Institute</t>
-        </is>
-      </c>
-      <c r="F12" s="37" t="inlineStr">
+      <c r="E12" s="44" t="inlineStr">
+        <is>
+          <t>Si Min Chan, NVIDIA; Masahiro Horibe, AIST G-QuAT; Dr Maggie Sou, Singapore Maritime Institute</t>
+        </is>
+      </c>
+      <c r="F12" s="44" t="inlineStr">
         <is>
           <t>Exploring autonomous AI agents that can reason, plan, collaborate, and make decisions in complex real-world environments.</t>
         </is>
@@ -976,14 +974,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C13" s="20" t="inlineStr">
+      <c r="C13" s="58" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="D13" s="20" t="n"/>
-      <c r="E13" s="20" t="n"/>
-      <c r="F13" s="20" t="n"/>
+      <c r="D13" s="58" t="n"/>
+      <c r="E13" s="58" t="n"/>
+      <c r="F13" s="58" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
@@ -996,22 +994,22 @@
           <t>SR12</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="C14" s="55" t="inlineStr">
         <is>
           <t>Quantum Computing for Risk Management</t>
         </is>
       </c>
-      <c r="D14" s="15" t="inlineStr">
+      <c r="D14" s="55" t="inlineStr">
         <is>
           <t>Paolo Giudici</t>
         </is>
       </c>
-      <c r="E14" s="15" t="inlineStr">
+      <c r="E14" s="55" t="inlineStr">
         <is>
           <t>Paolo Giudici</t>
         </is>
       </c>
-      <c r="F14" s="15" t="inlineStr">
+      <c r="F14" s="55" t="inlineStr">
         <is>
           <t>Safe AI Risk Management for Quantum AI</t>
         </is>
@@ -1040,14 +1038,14 @@
     <row r="15">
       <c r="A15" s="17" t="n"/>
       <c r="B15" s="19" t="n"/>
-      <c r="C15" s="20" t="n"/>
-      <c r="D15" s="20" t="n"/>
-      <c r="E15" s="20" t="inlineStr">
+      <c r="C15" s="58" t="n"/>
+      <c r="D15" s="58" t="n"/>
+      <c r="E15" s="58" t="inlineStr">
         <is>
           <t>Massimiliano Ferrera</t>
         </is>
       </c>
-      <c r="F15" s="20" t="inlineStr">
+      <c r="F15" s="58" t="inlineStr">
         <is>
           <t>Quantum Geometric Entropic Optimization</t>
         </is>
@@ -1056,14 +1054,14 @@
     <row r="16">
       <c r="A16" s="17" t="n"/>
       <c r="B16" s="19" t="n"/>
-      <c r="C16" s="20" t="n"/>
-      <c r="D16" s="20" t="n"/>
-      <c r="E16" s="20" t="inlineStr">
+      <c r="C16" s="58" t="n"/>
+      <c r="D16" s="58" t="n"/>
+      <c r="E16" s="58" t="inlineStr">
         <is>
           <t>Yash Rastogi</t>
         </is>
       </c>
-      <c r="F16" s="20" t="inlineStr">
+      <c r="F16" s="58" t="inlineStr">
         <is>
           <t>Quantum Computing for Bayesian Risk Analysis</t>
         </is>
@@ -1072,8 +1070,8 @@
     <row r="17">
       <c r="A17" s="17" t="n"/>
       <c r="B17" s="19" t="n"/>
-      <c r="C17" s="20" t="n"/>
-      <c r="D17" s="20" t="n"/>
+      <c r="C17" s="58" t="n"/>
+      <c r="D17" s="58" t="n"/>
       <c r="E17" s="31" t="inlineStr">
         <is>
           <t>Alessandro Bisio</t>
@@ -1096,22 +1094,22 @@
           <t>SR1</t>
         </is>
       </c>
-      <c r="C18" s="15" t="inlineStr">
+      <c r="C18" s="55" t="inlineStr">
         <is>
           <t>Advances in Bayesian Optimization &amp; Sequential Decision-Making</t>
         </is>
       </c>
-      <c r="D18" s="15" t="inlineStr">
+      <c r="D18" s="55" t="inlineStr">
         <is>
           <t>Ray-Bing Chen</t>
         </is>
       </c>
-      <c r="E18" s="15" t="inlineStr">
+      <c r="E18" s="55" t="inlineStr">
         <is>
           <t>Matthias Hwai-yong Tan</t>
         </is>
       </c>
-      <c r="F18" s="15" t="inlineStr">
+      <c r="F18" s="55" t="inlineStr">
         <is>
           <t>Computer Model Calibration via Bayesian Optimization Based on a Bi-Fidelity Gaussian Process Model for Transformed Sum of Squared Errors</t>
         </is>
@@ -1140,14 +1138,14 @@
     <row r="19">
       <c r="A19" s="17" t="n"/>
       <c r="B19" s="19" t="n"/>
-      <c r="C19" s="20" t="n"/>
-      <c r="D19" s="20" t="n"/>
-      <c r="E19" s="20" t="inlineStr">
+      <c r="C19" s="58" t="n"/>
+      <c r="D19" s="58" t="n"/>
+      <c r="E19" s="58" t="inlineStr">
         <is>
           <t>Wenjia Wang</t>
         </is>
       </c>
-      <c r="F19" s="20" t="inlineStr">
+      <c r="F19" s="58" t="inlineStr">
         <is>
           <t>SPARKLE: A Nonparametric Approach for Online Decision-Making with High-Dimensional Covariates</t>
         </is>
@@ -1156,14 +1154,14 @@
     <row r="20">
       <c r="A20" s="17" t="n"/>
       <c r="B20" s="19" t="n"/>
-      <c r="C20" s="20" t="n"/>
-      <c r="D20" s="20" t="n"/>
-      <c r="E20" s="20" t="inlineStr">
+      <c r="C20" s="58" t="n"/>
+      <c r="D20" s="58" t="n"/>
+      <c r="E20" s="58" t="inlineStr">
         <is>
           <t>Ping-Yang Chen</t>
         </is>
       </c>
-      <c r="F20" s="20" t="inlineStr">
+      <c r="F20" s="58" t="inlineStr">
         <is>
           <t>Bayesian Optimization for Mixed-Dimensional Inputs and Functional Outputs in Heat Treatment Process of Steel Manufacturing</t>
         </is>
@@ -1172,14 +1170,14 @@
     <row r="21">
       <c r="A21" s="17" t="n"/>
       <c r="B21" s="19" t="n"/>
-      <c r="C21" s="20" t="n"/>
-      <c r="D21" s="20" t="n"/>
-      <c r="E21" s="20" t="inlineStr">
+      <c r="C21" s="58" t="n"/>
+      <c r="D21" s="58" t="n"/>
+      <c r="E21" s="58" t="inlineStr">
         <is>
           <t>Ray-Bing Chen</t>
         </is>
       </c>
-      <c r="F21" s="20" t="inlineStr">
+      <c r="F21" s="58" t="inlineStr">
         <is>
           <t>Multi-Objective Bayesian Optimization of CPU Cooling Design with Mixed Variables Using Category Tree Gaussian Process</t>
         </is>
@@ -1196,22 +1194,22 @@
           <t>SR2</t>
         </is>
       </c>
-      <c r="C22" s="15" t="inlineStr">
+      <c r="C22" s="55" t="inlineStr">
         <is>
           <t>Exact Computation and Parallel Methods in Combinatorial Optimization</t>
         </is>
       </c>
-      <c r="D22" s="15" t="inlineStr">
+      <c r="D22" s="55" t="inlineStr">
         <is>
           <t>Koichi Fujii</t>
         </is>
       </c>
-      <c r="E22" s="15" t="inlineStr">
+      <c r="E22" s="55" t="inlineStr">
         <is>
           <t>Koichi Fujii</t>
         </is>
       </c>
-      <c r="F22" s="15" t="inlineStr">
+      <c r="F22" s="55" t="inlineStr">
         <is>
           <t>From Computation to Proof: Experiments with QAP and Circle Graphs</t>
         </is>
@@ -1240,14 +1238,14 @@
     <row r="23">
       <c r="A23" s="17" t="n"/>
       <c r="B23" s="19" t="n"/>
-      <c r="C23" s="20" t="n"/>
-      <c r="D23" s="20" t="n"/>
-      <c r="E23" s="20" t="inlineStr">
+      <c r="C23" s="58" t="n"/>
+      <c r="D23" s="58" t="n"/>
+      <c r="E23" s="58" t="inlineStr">
         <is>
           <t>Hirotaka Ono</t>
         </is>
       </c>
-      <c r="F23" s="20" t="inlineStr">
+      <c r="F23" s="58" t="inlineStr">
         <is>
           <t>Exact Depths and Bounds for Small Selection Networks</t>
         </is>
@@ -1256,14 +1254,14 @@
     <row r="24">
       <c r="A24" s="17" t="n"/>
       <c r="B24" s="19" t="n"/>
-      <c r="C24" s="20" t="n"/>
-      <c r="D24" s="20" t="n"/>
-      <c r="E24" s="20" t="inlineStr">
+      <c r="C24" s="58" t="n"/>
+      <c r="D24" s="58" t="n"/>
+      <c r="E24" s="58" t="inlineStr">
         <is>
           <t>Yuji Shinano</t>
         </is>
       </c>
-      <c r="F24" s="20" t="inlineStr">
+      <c r="F24" s="58" t="inlineStr">
         <is>
           <t>Exploiting the Diversity of State-of-the-Art MIP Solvers in Parallel</t>
         </is>
@@ -1272,14 +1270,14 @@
     <row r="25">
       <c r="A25" s="17" t="n"/>
       <c r="B25" s="19" t="n"/>
-      <c r="C25" s="20" t="n"/>
-      <c r="D25" s="20" t="n"/>
-      <c r="E25" s="20" t="inlineStr">
+      <c r="C25" s="58" t="n"/>
+      <c r="D25" s="58" t="n"/>
+      <c r="E25" s="58" t="inlineStr">
         <is>
           <t>JingFeng Yang</t>
         </is>
       </c>
-      <c r="F25" s="20" t="inlineStr">
+      <c r="F25" s="58" t="inlineStr">
         <is>
           <t>GenAI Meets Mathematical Optimization: Lessons and Opportunities from the Gurobi Intelligence Hub</t>
         </is>
@@ -1296,22 +1294,22 @@
           <t>SR3</t>
         </is>
       </c>
-      <c r="C26" s="15" t="inlineStr">
+      <c r="C26" s="55" t="inlineStr">
         <is>
           <t>Mathematical Foundation of Quantum Computing</t>
         </is>
       </c>
-      <c r="D26" s="15" t="inlineStr">
+      <c r="D26" s="55" t="inlineStr">
         <is>
           <t>Josef Teichmann</t>
         </is>
       </c>
-      <c r="E26" s="15" t="inlineStr">
+      <c r="E26" s="55" t="inlineStr">
         <is>
           <t>Hoang Vu</t>
         </is>
       </c>
-      <c r="F26" s="15" t="inlineStr">
+      <c r="F26" s="55" t="inlineStr">
         <is>
           <t>A Probabilistic Representation for Multi-State Discrete-Time
 Quantum Walks</t>
@@ -1341,9 +1339,9 @@
     <row r="27">
       <c r="A27" s="17" t="n"/>
       <c r="B27" s="19" t="n"/>
-      <c r="C27" s="20" t="n"/>
-      <c r="D27" s="20" t="n"/>
-      <c r="E27" s="20" t="inlineStr">
+      <c r="C27" s="58" t="n"/>
+      <c r="D27" s="58" t="n"/>
+      <c r="E27" s="58" t="inlineStr">
         <is>
           <t>Ege Yilmaz</t>
         </is>
@@ -1357,9 +1355,9 @@
     <row r="28">
       <c r="A28" s="17" t="n"/>
       <c r="B28" s="19" t="n"/>
-      <c r="C28" s="20" t="n"/>
-      <c r="D28" s="20" t="n"/>
-      <c r="E28" s="20" t="inlineStr">
+      <c r="C28" s="58" t="n"/>
+      <c r="D28" s="58" t="n"/>
+      <c r="E28" s="58" t="inlineStr">
         <is>
           <t>Ariel Neufeld</t>
         </is>
@@ -1373,14 +1371,14 @@
     <row r="29">
       <c r="A29" s="17" t="n"/>
       <c r="B29" s="19" t="n"/>
-      <c r="C29" s="20" t="n"/>
-      <c r="D29" s="20" t="n"/>
-      <c r="E29" s="20" t="inlineStr">
+      <c r="C29" s="58" t="n"/>
+      <c r="D29" s="58" t="n"/>
+      <c r="E29" s="58" t="inlineStr">
         <is>
           <t>Josef Teichmann</t>
         </is>
       </c>
-      <c r="F29" s="20" t="inlineStr">
+      <c r="F29" s="58" t="inlineStr">
         <is>
           <t>A universality result in Quantum Reservoir Computing</t>
         </is>
@@ -1393,14 +1391,14 @@
           <t>SR4</t>
         </is>
       </c>
-      <c r="C30" s="20" t="n"/>
-      <c r="D30" s="20" t="n"/>
+      <c r="C30" s="58" t="n"/>
+      <c r="D30" s="58" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="17" t="n"/>
       <c r="B31" s="19" t="n"/>
-      <c r="C31" s="20" t="n"/>
-      <c r="D31" s="20" t="n"/>
+      <c r="C31" s="58" t="n"/>
+      <c r="D31" s="58" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="36" t="inlineStr">
@@ -1643,12 +1641,12 @@
       <c r="B38" s="57" t="n"/>
       <c r="C38" s="58" t="n"/>
       <c r="D38" s="58" t="n"/>
-      <c r="E38" s="59" t="inlineStr">
+      <c r="E38" s="61" t="inlineStr">
         <is>
           <t>Jianlong Lu</t>
         </is>
       </c>
-      <c r="F38" s="59" t="inlineStr">
+      <c r="F38" s="61" t="inlineStr">
         <is>
           <t>Beyond Hardware: Adaptive Algorithmic Control by State-Proxy Equalization</t>
         </is>
@@ -1757,8 +1755,8 @@
     <row r="43">
       <c r="A43" s="17" t="n"/>
       <c r="B43" s="19" t="n"/>
-      <c r="C43" s="20" t="n"/>
-      <c r="D43" s="20" t="n"/>
+      <c r="C43" s="58" t="n"/>
+      <c r="D43" s="58" t="n"/>
       <c r="E43" s="22" t="n"/>
       <c r="F43" s="22" t="n"/>
     </row>
@@ -1773,22 +1771,22 @@
           <t>SR1</t>
         </is>
       </c>
-      <c r="C44" s="15" t="inlineStr">
+      <c r="C44" s="55" t="inlineStr">
         <is>
           <t>Modern Methods in Statistical Modeling &amp; Inference</t>
         </is>
       </c>
-      <c r="D44" s="15" t="inlineStr">
+      <c r="D44" s="55" t="inlineStr">
         <is>
           <t>Takayuki Shiohama</t>
         </is>
       </c>
-      <c r="E44" s="15" t="inlineStr">
+      <c r="E44" s="55" t="inlineStr">
         <is>
           <t>Takato Hashino</t>
         </is>
       </c>
-      <c r="F44" s="15" t="inlineStr">
+      <c r="F44" s="55" t="inlineStr">
         <is>
           <t>Estimating the Shannon Entropy Using the Pitman–Yor Process</t>
         </is>
@@ -1817,14 +1815,14 @@
     <row r="45">
       <c r="A45" s="17" t="n"/>
       <c r="B45" s="19" t="n"/>
-      <c r="C45" s="20" t="n"/>
-      <c r="D45" s="20" t="n"/>
-      <c r="E45" s="20" t="inlineStr">
+      <c r="C45" s="58" t="n"/>
+      <c r="D45" s="58" t="n"/>
+      <c r="E45" s="58" t="inlineStr">
         <is>
           <t>Kohei Kawamoto</t>
         </is>
       </c>
-      <c r="F45" s="20" t="inlineStr">
+      <c r="F45" s="58" t="inlineStr">
         <is>
           <t>High-Dimensional Theory of PCA Connectivity Analysis for Three-Group Mixtures</t>
         </is>
@@ -1833,14 +1831,14 @@
     <row r="46">
       <c r="A46" s="17" t="n"/>
       <c r="B46" s="19" t="n"/>
-      <c r="C46" s="20" t="n"/>
-      <c r="D46" s="20" t="n"/>
-      <c r="E46" s="20" t="inlineStr">
+      <c r="C46" s="58" t="n"/>
+      <c r="D46" s="58" t="n"/>
+      <c r="E46" s="58" t="inlineStr">
         <is>
           <t>Tomoaki Imoto</t>
         </is>
       </c>
-      <c r="F46" s="20" t="inlineStr">
+      <c r="F46" s="58" t="inlineStr">
         <is>
           <t>Proposition of New Toroidal Distribution: Bivariate Extended Wrapped Cauchy Distribution</t>
         </is>
@@ -1849,14 +1847,14 @@
     <row r="47">
       <c r="A47" s="17" t="n"/>
       <c r="B47" s="19" t="n"/>
-      <c r="C47" s="20" t="n"/>
-      <c r="D47" s="20" t="n"/>
-      <c r="E47" s="20" t="inlineStr">
+      <c r="C47" s="58" t="n"/>
+      <c r="D47" s="58" t="n"/>
+      <c r="E47" s="58" t="inlineStr">
         <is>
           <t>Junichi Hirukawa</t>
         </is>
       </c>
-      <c r="F47" s="20" t="inlineStr">
+      <c r="F47" s="58" t="inlineStr">
         <is>
           <t>The Second-Order Generalization of Hájek–Le Cam Asymptotic Minimax Theorem</t>
         </is>
@@ -1873,12 +1871,12 @@
           <t>SR2</t>
         </is>
       </c>
-      <c r="C48" s="15" t="inlineStr">
+      <c r="C48" s="55" t="inlineStr">
         <is>
           <t>Industrial Deployment of AI: From Algorithmic Innovation to Production Realities</t>
         </is>
       </c>
-      <c r="D48" s="15" t="inlineStr">
+      <c r="D48" s="55" t="inlineStr">
         <is>
           <t>Dennis Thumm</t>
         </is>
@@ -1917,8 +1915,8 @@
     <row r="49">
       <c r="A49" s="17" t="n"/>
       <c r="B49" s="19" t="n"/>
-      <c r="C49" s="20" t="n"/>
-      <c r="D49" s="20" t="n"/>
+      <c r="C49" s="58" t="n"/>
+      <c r="D49" s="58" t="n"/>
       <c r="E49" s="61" t="inlineStr">
         <is>
           <t>Marvin Carl May</t>
@@ -1933,8 +1931,8 @@
     <row r="50">
       <c r="A50" s="17" t="n"/>
       <c r="B50" s="19" t="n"/>
-      <c r="C50" s="20" t="n"/>
-      <c r="D50" s="20" t="n"/>
+      <c r="C50" s="58" t="n"/>
+      <c r="D50" s="58" t="n"/>
       <c r="E50" s="61" t="inlineStr">
         <is>
           <t>Hsing Sung Tsai</t>
@@ -1949,8 +1947,8 @@
     <row r="51">
       <c r="A51" s="17" t="n"/>
       <c r="B51" s="19" t="n"/>
-      <c r="C51" s="20" t="n"/>
-      <c r="D51" s="20" t="n"/>
+      <c r="C51" s="58" t="n"/>
+      <c r="D51" s="58" t="n"/>
       <c r="E51" s="32" t="inlineStr">
         <is>
           <t>Maris T. Lasco</t>
@@ -1973,12 +1971,12 @@
           <t>SR3</t>
         </is>
       </c>
-      <c r="C52" s="15" t="inlineStr">
+      <c r="C52" s="55" t="inlineStr">
         <is>
           <t>Advances in Quantum Computing and AI Applications</t>
         </is>
       </c>
-      <c r="D52" s="15" t="inlineStr">
+      <c r="D52" s="55" t="inlineStr">
         <is>
           <t>Ralf Borndörfer</t>
         </is>
@@ -2017,8 +2015,8 @@
     <row r="53">
       <c r="A53" s="17" t="n"/>
       <c r="B53" s="19" t="n"/>
-      <c r="C53" s="20" t="n"/>
-      <c r="D53" s="20" t="n"/>
+      <c r="C53" s="58" t="n"/>
+      <c r="D53" s="58" t="n"/>
       <c r="E53" s="32" t="inlineStr">
         <is>
           <t>Mrinal Kanti Giri</t>
@@ -2033,8 +2031,8 @@
     <row r="54">
       <c r="A54" s="17" t="n"/>
       <c r="B54" s="19" t="n"/>
-      <c r="C54" s="20" t="n"/>
-      <c r="D54" s="20" t="n"/>
+      <c r="C54" s="58" t="n"/>
+      <c r="D54" s="58" t="n"/>
       <c r="E54" s="32" t="inlineStr">
         <is>
           <t>Yuting Zhu</t>
@@ -2049,8 +2047,8 @@
     <row r="55">
       <c r="A55" s="17" t="n"/>
       <c r="B55" s="19" t="n"/>
-      <c r="C55" s="20" t="n"/>
-      <c r="D55" s="20" t="n"/>
+      <c r="C55" s="58" t="n"/>
+      <c r="D55" s="58" t="n"/>
       <c r="E55" s="32" t="inlineStr">
         <is>
           <t>Gloria Wu</t>
@@ -2083,12 +2081,12 @@
           <t>Patrick Rebentrost</t>
         </is>
       </c>
-      <c r="E56" s="15" t="inlineStr">
+      <c r="E56" s="55" t="inlineStr">
         <is>
           <t>Dong-Ling Deng (Tsinghua)</t>
         </is>
       </c>
-      <c r="F56" s="15" t="inlineStr">
+      <c r="F56" s="55" t="inlineStr">
         <is>
           <t>Quantum Artificial Intelligence: The Endless Frontier</t>
         </is>
@@ -2115,12 +2113,12 @@
       <c r="B58" s="62" t="n"/>
       <c r="C58" s="62" t="n"/>
       <c r="D58" s="62" t="n"/>
-      <c r="E58" s="20" t="inlineStr">
+      <c r="E58" s="58" t="inlineStr">
         <is>
           <t>Wei Wang (Hong Kong Polytechnic University)</t>
         </is>
       </c>
-      <c r="F58" s="20" t="inlineStr">
+      <c r="F58" s="58" t="inlineStr">
         <is>
           <t>Leveraging Loss Tolerance in Photonic Quantum Microprocessors for Large-Scale Combinatorial Optimization</t>
         </is>
@@ -2131,12 +2129,12 @@
       <c r="B59" s="62" t="n"/>
       <c r="C59" s="62" t="n"/>
       <c r="D59" s="62" t="n"/>
-      <c r="E59" s="20" t="inlineStr">
+      <c r="E59" s="58" t="inlineStr">
         <is>
           <t>Patrick Rebentrost group/Naixu Guo</t>
         </is>
       </c>
-      <c r="F59" s="20" t="inlineStr">
+      <c r="F59" s="58" t="inlineStr">
         <is>
           <t>Quantum computing for derivative pricing/AI for designing quantum algorithms.</t>
         </is>
@@ -2151,20 +2149,20 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C60" s="20" t="inlineStr">
+      <c r="C60" s="58" t="inlineStr">
         <is>
           <t>End of Day 1</t>
         </is>
       </c>
-      <c r="D60" s="20" t="n"/>
-      <c r="E60" s="20" t="n"/>
-      <c r="F60" s="20" t="n"/>
+      <c r="D60" s="58" t="n"/>
+      <c r="E60" s="58" t="n"/>
+      <c r="F60" s="58" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="48" t="n"/>
       <c r="B61" s="19" t="n"/>
-      <c r="C61" s="20" t="n"/>
-      <c r="D61" s="20" t="n"/>
+      <c r="C61" s="58" t="n"/>
+      <c r="D61" s="58" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2232,22 +2230,22 @@
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="51" t="inlineStr">
         <is>
           <t>Keynote 3</t>
         </is>
       </c>
-      <c r="D2" s="18" t="inlineStr">
+      <c r="D2" s="52" t="inlineStr">
         <is>
           <t>Chair: Thorsten Koch</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E2" s="51" t="inlineStr">
         <is>
           <t>Simon See, NVIDIA</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F2" s="51" t="inlineStr">
         <is>
           <t>From Language to Reality: The Road from Foundation Models to World Models and Quantum Computing</t>
         </is>
@@ -2284,14 +2282,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C3" s="20" t="inlineStr">
+      <c r="C3" s="58" t="inlineStr">
         <is>
           <t>Tea Break</t>
         </is>
       </c>
-      <c r="D3" s="20" t="n"/>
-      <c r="E3" s="20" t="n"/>
-      <c r="F3" s="20" t="n"/>
+      <c r="D3" s="58" t="n"/>
+      <c r="E3" s="58" t="n"/>
+      <c r="F3" s="58" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
@@ -2304,22 +2302,22 @@
           <t>SR12</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C4" s="55" t="inlineStr">
         <is>
           <t>Advanced Optimization, Vision &amp; LLMs</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="D4" s="55" t="inlineStr">
         <is>
           <t>Katsuki Fujisawa</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="55" t="inlineStr">
         <is>
           <t>Katsuki Fujisawa</t>
         </is>
       </c>
-      <c r="F4" s="15" t="inlineStr">
+      <c r="F4" s="55" t="inlineStr">
         <is>
           <t>Intelligent Manufacturing and Mobility Optimization: Integrating Deep Learning, LLMs, and Quantum Computing</t>
         </is>
@@ -2348,14 +2346,14 @@
     <row r="5">
       <c r="A5" s="17" t="n"/>
       <c r="B5" s="19" t="n"/>
-      <c r="C5" s="20" t="n"/>
-      <c r="D5" s="20" t="n"/>
-      <c r="E5" s="20" t="inlineStr">
+      <c r="C5" s="58" t="n"/>
+      <c r="D5" s="58" t="n"/>
+      <c r="E5" s="58" t="inlineStr">
         <is>
           <t>Yoshihiko Fujisawa</t>
         </is>
       </c>
-      <c r="F5" s="20" t="inlineStr">
+      <c r="F5" s="58" t="inlineStr">
         <is>
           <t>More Than Bits: Multi-Envelope Double Binary Factorization for Extreme Quantization of Large Language Models</t>
         </is>
@@ -2364,14 +2362,14 @@
     <row r="6">
       <c r="A6" s="17" t="n"/>
       <c r="B6" s="19" t="n"/>
-      <c r="C6" s="20" t="n"/>
-      <c r="D6" s="20" t="n"/>
-      <c r="E6" s="20" t="inlineStr">
+      <c r="C6" s="58" t="n"/>
+      <c r="D6" s="58" t="n"/>
+      <c r="E6" s="58" t="inlineStr">
         <is>
           <t>Ken Kawano</t>
         </is>
       </c>
-      <c r="F6" s="20" t="inlineStr">
+      <c r="F6" s="58" t="inlineStr">
         <is>
           <t>Localization-Confidence-Aware Pseudo-Label Selection for Semi-Supervised Object Detection</t>
         </is>
@@ -2380,8 +2378,8 @@
     <row r="7">
       <c r="A7" s="17" t="n"/>
       <c r="B7" s="19" t="n"/>
-      <c r="C7" s="20" t="n"/>
-      <c r="D7" s="20" t="n"/>
+      <c r="C7" s="58" t="n"/>
+      <c r="D7" s="58" t="n"/>
       <c r="E7" s="22" t="n"/>
       <c r="F7" s="22" t="n"/>
     </row>
@@ -2396,22 +2394,22 @@
           <t>SR1</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="C8" s="55" t="inlineStr">
         <is>
           <t>Reservoir Computing &amp; Dynamics Learning</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="D8" s="55" t="inlineStr">
         <is>
           <t>Juan-Pablo Ortega &amp; Florian Rossmannek</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
+      <c r="E8" s="55" t="inlineStr">
         <is>
           <t>Thiparat Chotibut</t>
         </is>
       </c>
-      <c r="F8" s="15" t="inlineStr">
+      <c r="F8" s="55" t="inlineStr">
         <is>
           <t>Roles of Scrambling and Noise in Information Processing with Quantum Systems</t>
         </is>
@@ -2440,14 +2438,14 @@
     <row r="9">
       <c r="A9" s="17" t="n"/>
       <c r="B9" s="19" t="n"/>
-      <c r="C9" s="20" t="n"/>
-      <c r="D9" s="20" t="n"/>
-      <c r="E9" s="20" t="inlineStr">
+      <c r="C9" s="58" t="n"/>
+      <c r="D9" s="58" t="n"/>
+      <c r="E9" s="58" t="inlineStr">
         <is>
           <t>Tomoyuki Kubota</t>
         </is>
       </c>
-      <c r="F9" s="20" t="inlineStr">
+      <c r="F9" s="58" t="inlineStr">
         <is>
           <t>Utilizing Quantum Noise for Temporal Information Processing</t>
         </is>
@@ -2456,14 +2454,14 @@
     <row r="10">
       <c r="A10" s="17" t="n"/>
       <c r="B10" s="19" t="n"/>
-      <c r="C10" s="20" t="n"/>
-      <c r="D10" s="20" t="n"/>
-      <c r="E10" s="20" t="inlineStr">
+      <c r="C10" s="58" t="n"/>
+      <c r="D10" s="58" t="n"/>
+      <c r="E10" s="58" t="inlineStr">
         <is>
           <t>Jianyu Hu</t>
         </is>
       </c>
-      <c r="F10" s="20" t="inlineStr">
+      <c r="F10" s="58" t="inlineStr">
         <is>
           <t>Kernel Learning of PDE Solution Operators</t>
         </is>
@@ -2472,14 +2470,14 @@
     <row r="11">
       <c r="A11" s="17" t="n"/>
       <c r="B11" s="19" t="n"/>
-      <c r="C11" s="20" t="n"/>
-      <c r="D11" s="20" t="n"/>
-      <c r="E11" s="20" t="inlineStr">
+      <c r="C11" s="58" t="n"/>
+      <c r="D11" s="58" t="n"/>
+      <c r="E11" s="58" t="inlineStr">
         <is>
           <t>Florian Rossmannek</t>
         </is>
       </c>
-      <c r="F11" s="20" t="inlineStr">
+      <c r="F11" s="58" t="inlineStr">
         <is>
           <t>State-Space and State-Affine Systems for Learning from Temporal Data</t>
         </is>
@@ -2496,22 +2494,22 @@
           <t>SR2</t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr">
+      <c r="C12" s="55" t="inlineStr">
         <is>
           <t>Reliable &amp; Adaptive AI</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
+      <c r="D12" s="55" t="inlineStr">
         <is>
           <t>Chuan-Ju Wang</t>
         </is>
       </c>
-      <c r="E12" s="15" t="inlineStr">
+      <c r="E12" s="55" t="inlineStr">
         <is>
           <t>Chuan-Ju Wang</t>
         </is>
       </c>
-      <c r="F12" s="15" t="inlineStr">
+      <c r="F12" s="55" t="inlineStr">
         <is>
           <t>Numerically Aware and Reliable Language Understanding: Toward Trustworthy AI for Financial Intelligence</t>
         </is>
@@ -2540,14 +2538,14 @@
     <row r="13">
       <c r="A13" s="17" t="n"/>
       <c r="B13" s="19" t="n"/>
-      <c r="C13" s="20" t="n"/>
-      <c r="D13" s="20" t="n"/>
-      <c r="E13" s="20" t="inlineStr">
+      <c r="C13" s="58" t="n"/>
+      <c r="D13" s="58" t="n"/>
+      <c r="E13" s="58" t="inlineStr">
         <is>
           <t>Hen-Hsen Huang</t>
         </is>
       </c>
-      <c r="F13" s="20" t="inlineStr">
+      <c r="F13" s="58" t="inlineStr">
         <is>
           <t>Trustworthy Local LLMs: Building Under Data, Resource, and Supervision Constraints</t>
         </is>
@@ -2556,14 +2554,14 @@
     <row r="14">
       <c r="A14" s="17" t="n"/>
       <c r="B14" s="19" t="n"/>
-      <c r="C14" s="20" t="n"/>
-      <c r="D14" s="20" t="n"/>
-      <c r="E14" s="20" t="inlineStr">
+      <c r="C14" s="58" t="n"/>
+      <c r="D14" s="58" t="n"/>
+      <c r="E14" s="58" t="inlineStr">
         <is>
           <t>Yun-Hsuan Lien</t>
         </is>
       </c>
-      <c r="F14" s="20" t="inlineStr">
+      <c r="F14" s="58" t="inlineStr">
         <is>
           <t>Adaptive and Reliable Reinforcement Learning: Toward Human-Centered Embodied Intelligence</t>
         </is>
@@ -2572,14 +2570,14 @@
     <row r="15">
       <c r="A15" s="17" t="n"/>
       <c r="B15" s="19" t="n"/>
-      <c r="C15" s="20" t="n"/>
-      <c r="D15" s="20" t="n"/>
-      <c r="E15" s="20" t="inlineStr">
+      <c r="C15" s="58" t="n"/>
+      <c r="D15" s="58" t="n"/>
+      <c r="E15" s="58" t="inlineStr">
         <is>
           <t>Yu-Hsi Chen; Wei-Hsin Chen</t>
         </is>
       </c>
-      <c r="F15" s="20" t="inlineStr">
+      <c r="F15" s="58" t="inlineStr">
         <is>
           <t>Deep Learning-Based Analysis of Spontaneous Behavior Enables Early Detection of Alzheimer's Disease in Mouse Models</t>
         </is>
@@ -2596,22 +2594,22 @@
           <t>SR3</t>
         </is>
       </c>
-      <c r="C16" s="15" t="inlineStr">
+      <c r="C16" s="55" t="inlineStr">
         <is>
           <t>Statistical &amp; Network Modeling of Knowledge Discovery and Scientific Systems</t>
         </is>
       </c>
-      <c r="D16" s="15" t="inlineStr">
+      <c r="D16" s="55" t="inlineStr">
         <is>
           <t>Frederick Kin Hing Phoa</t>
         </is>
       </c>
-      <c r="E16" s="15" t="inlineStr">
+      <c r="E16" s="55" t="inlineStr">
         <is>
           <t>Wen Han Gao</t>
         </is>
       </c>
-      <c r="F16" s="15" t="inlineStr">
+      <c r="F16" s="55" t="inlineStr">
         <is>
           <t>Innovation Value Discrepancy: Impact on Short-Term Gains and Sustainable Growth</t>
         </is>
@@ -2640,14 +2638,14 @@
     <row r="17">
       <c r="A17" s="17" t="n"/>
       <c r="B17" s="19" t="n"/>
-      <c r="C17" s="20" t="n"/>
-      <c r="D17" s="20" t="n"/>
-      <c r="E17" s="20" t="inlineStr">
+      <c r="C17" s="58" t="n"/>
+      <c r="D17" s="58" t="n"/>
+      <c r="E17" s="58" t="inlineStr">
         <is>
           <t>Tzu-Yin Chen</t>
         </is>
       </c>
-      <c r="F17" s="20" t="inlineStr">
+      <c r="F17" s="58" t="inlineStr">
         <is>
           <t>Modeling Academic Collaboration Networks Using Hypergraph Theory: A Large-Scale Scientometric Analysis of Scopus Data</t>
         </is>
@@ -2656,9 +2654,9 @@
     <row r="18">
       <c r="A18" s="17" t="n"/>
       <c r="B18" s="19" t="n"/>
-      <c r="C18" s="20" t="n"/>
-      <c r="D18" s="20" t="n"/>
-      <c r="E18" s="20" t="inlineStr">
+      <c r="C18" s="58" t="n"/>
+      <c r="D18" s="58" t="n"/>
+      <c r="E18" s="58" t="inlineStr">
         <is>
           <t>Yuji Mizukami</t>
         </is>
@@ -2672,14 +2670,14 @@
     <row r="19">
       <c r="A19" s="17" t="n"/>
       <c r="B19" s="19" t="n"/>
-      <c r="C19" s="20" t="n"/>
-      <c r="D19" s="20" t="n"/>
-      <c r="E19" s="20" t="inlineStr">
+      <c r="C19" s="58" t="n"/>
+      <c r="D19" s="58" t="n"/>
+      <c r="E19" s="58" t="inlineStr">
         <is>
           <t>Frederick Kin Hing Phoa</t>
         </is>
       </c>
-      <c r="F19" s="20" t="inlineStr">
+      <c r="F19" s="58" t="inlineStr">
         <is>
           <t>Mapping Citation Tendencies among Broad Subject Groups: Closed Fields, Asymmetric Exchange, Unexpected Ties and Structural Disconnection</t>
         </is>
@@ -2696,22 +2694,22 @@
           <t>SR4</t>
         </is>
       </c>
-      <c r="C20" s="15" t="inlineStr">
+      <c r="C20" s="55" t="inlineStr">
         <is>
           <t>Trustworthy Machine Learning with Applications</t>
         </is>
       </c>
-      <c r="D20" s="15" t="inlineStr">
+      <c r="D20" s="55" t="inlineStr">
         <is>
           <t>Henry Horng-Shing Lu</t>
         </is>
       </c>
-      <c r="E20" s="15" t="inlineStr">
+      <c r="E20" s="55" t="inlineStr">
         <is>
           <t>Grace Hyun J. Kim</t>
         </is>
       </c>
-      <c r="F20" s="15" t="inlineStr">
+      <c r="F20" s="55" t="inlineStr">
         <is>
           <t>Deep Learning-Based Fibrosis Scoring from High Resolution Computed Tomography</t>
         </is>
@@ -2740,14 +2738,14 @@
     <row r="21">
       <c r="A21" s="17" t="n"/>
       <c r="B21" s="19" t="n"/>
-      <c r="C21" s="20" t="n"/>
-      <c r="D21" s="20" t="n"/>
-      <c r="E21" s="20" t="inlineStr">
+      <c r="C21" s="58" t="n"/>
+      <c r="D21" s="58" t="n"/>
+      <c r="E21" s="58" t="inlineStr">
         <is>
           <t>Guan-Ju Peng</t>
         </is>
       </c>
-      <c r="F21" s="20" t="inlineStr">
+      <c r="F21" s="58" t="inlineStr">
         <is>
           <t>From Predictions to Executable Portfolios: Sparse Signals, Adaptive Support, and Reliability-Weighted Policy Composition</t>
         </is>
@@ -2756,14 +2754,14 @@
     <row r="22">
       <c r="A22" s="17" t="n"/>
       <c r="B22" s="19" t="n"/>
-      <c r="C22" s="20" t="n"/>
-      <c r="D22" s="20" t="n"/>
-      <c r="E22" s="20" t="inlineStr">
+      <c r="C22" s="58" t="n"/>
+      <c r="D22" s="58" t="n"/>
+      <c r="E22" s="58" t="inlineStr">
         <is>
           <t>Kani Chen</t>
         </is>
       </c>
-      <c r="F22" s="20" t="inlineStr">
+      <c r="F22" s="58" t="inlineStr">
         <is>
           <t>Quantifying Fidelity in Agentic AI: Statistical Foundations of Personality Alignment and Demographic Inference</t>
         </is>
@@ -2772,14 +2770,14 @@
     <row r="23">
       <c r="A23" s="17" t="n"/>
       <c r="B23" s="19" t="n"/>
-      <c r="C23" s="20" t="n"/>
-      <c r="D23" s="20" t="n"/>
-      <c r="E23" s="20" t="inlineStr">
+      <c r="C23" s="58" t="n"/>
+      <c r="D23" s="58" t="n"/>
+      <c r="E23" s="58" t="inlineStr">
         <is>
           <t>Henry Horng-Shing Lu</t>
         </is>
       </c>
-      <c r="F23" s="20" t="inlineStr">
+      <c r="F23" s="58" t="inlineStr">
         <is>
           <t>Test-Fairness Deep Learning with Influence Score</t>
         </is>
@@ -2796,18 +2794,18 @@
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C24" s="24" t="inlineStr">
+      <c r="C24" s="40" t="inlineStr">
         <is>
           <t>Showcase 3</t>
         </is>
       </c>
-      <c r="D24" s="24" t="n"/>
-      <c r="E24" s="24" t="inlineStr">
+      <c r="D24" s="40" t="n"/>
+      <c r="E24" s="40" t="inlineStr">
         <is>
           <t>Matthias W. Uhl, Managing Director, UBS Asset Management</t>
         </is>
       </c>
-      <c r="F24" s="24" t="inlineStr">
+      <c r="F24" s="40" t="inlineStr">
         <is>
           <t>AI in the Investment Process of a Global Asset Manager</t>
         </is>
@@ -2844,17 +2842,17 @@
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C25" s="37" t="inlineStr">
+      <c r="C25" s="44" t="inlineStr">
         <is>
           <t>Panel 3: Quantum × AI for Finance and Risk</t>
         </is>
       </c>
-      <c r="D25" s="37" t="inlineStr">
+      <c r="D25" s="44" t="inlineStr">
         <is>
           <t>Moderator: Paolo Giudici</t>
         </is>
       </c>
-      <c r="E25" s="37" t="inlineStr">
+      <c r="E25" s="44" t="inlineStr">
         <is>
           <t>Huaxing Chen, UOB/NUS; Matthias W. Uhl, UBS; Stefan Woerner, IBM Research Europe – Zurich</t>
         </is>
@@ -2892,14 +2890,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C26" s="20" t="inlineStr">
+      <c r="C26" s="58" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="D26" s="20" t="n"/>
-      <c r="E26" s="20" t="n"/>
-      <c r="F26" s="20" t="n"/>
+      <c r="D26" s="58" t="n"/>
+      <c r="E26" s="58" t="n"/>
+      <c r="F26" s="58" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
@@ -2912,18 +2910,18 @@
           <t>SR12</t>
         </is>
       </c>
-      <c r="C27" s="20" t="inlineStr">
+      <c r="C27" s="58" t="inlineStr">
         <is>
           <t>Hands-on 1: Agentic AI Coding</t>
         </is>
       </c>
-      <c r="D27" s="20" t="inlineStr">
+      <c r="D27" s="58" t="inlineStr">
         <is>
           <t>Thorsten Koch</t>
         </is>
       </c>
-      <c r="E27" s="20" t="n"/>
-      <c r="F27" s="20" t="inlineStr">
+      <c r="E27" s="58" t="n"/>
+      <c r="F27" s="58" t="inlineStr">
         <is>
           <t>Part I</t>
         </is>
@@ -2940,18 +2938,18 @@
           <t>SR1</t>
         </is>
       </c>
-      <c r="C28" s="20" t="inlineStr">
+      <c r="C28" s="58" t="inlineStr">
         <is>
           <t>Hands-on 2: Quantum Computing</t>
         </is>
       </c>
-      <c r="D28" s="20" t="inlineStr">
+      <c r="D28" s="58" t="inlineStr">
         <is>
           <t>Vishal Bajpe</t>
         </is>
       </c>
-      <c r="E28" s="20" t="n"/>
-      <c r="F28" s="20" t="inlineStr">
+      <c r="E28" s="58" t="n"/>
+      <c r="F28" s="58" t="inlineStr">
         <is>
           <t>Part I</t>
         </is>
@@ -2968,14 +2966,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C29" s="20" t="inlineStr">
+      <c r="C29" s="58" t="inlineStr">
         <is>
           <t>Tea Break</t>
         </is>
       </c>
-      <c r="D29" s="20" t="n"/>
-      <c r="E29" s="20" t="n"/>
-      <c r="F29" s="20" t="n"/>
+      <c r="D29" s="58" t="n"/>
+      <c r="E29" s="58" t="n"/>
+      <c r="F29" s="58" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
@@ -2988,18 +2986,18 @@
           <t>SR12</t>
         </is>
       </c>
-      <c r="C30" s="20" t="inlineStr">
+      <c r="C30" s="58" t="inlineStr">
         <is>
           <t>Hands-on 1: Agentic AI Coding</t>
         </is>
       </c>
-      <c r="D30" s="20" t="inlineStr">
+      <c r="D30" s="58" t="inlineStr">
         <is>
           <t>Thorsten Koch</t>
         </is>
       </c>
-      <c r="E30" s="20" t="n"/>
-      <c r="F30" s="20" t="inlineStr">
+      <c r="E30" s="58" t="n"/>
+      <c r="F30" s="58" t="inlineStr">
         <is>
           <t>Part II</t>
         </is>
@@ -3016,18 +3014,18 @@
           <t>SR1</t>
         </is>
       </c>
-      <c r="C31" s="20" t="inlineStr">
+      <c r="C31" s="58" t="inlineStr">
         <is>
           <t>Hands-on 2: Quantum Computing</t>
         </is>
       </c>
-      <c r="D31" s="20" t="inlineStr">
+      <c r="D31" s="58" t="inlineStr">
         <is>
           <t>Vishal Bajpe</t>
         </is>
       </c>
-      <c r="E31" s="20" t="n"/>
-      <c r="F31" s="20" t="inlineStr">
+      <c r="E31" s="58" t="n"/>
+      <c r="F31" s="58" t="inlineStr">
         <is>
           <t>Part II</t>
         </is>
@@ -3038,14 +3036,14 @@
         <v>0.7083333333333334</v>
       </c>
       <c r="B32" s="19" t="n"/>
-      <c r="C32" s="20" t="inlineStr">
+      <c r="C32" s="58" t="inlineStr">
         <is>
           <t>End of Day 2</t>
         </is>
       </c>
-      <c r="D32" s="20" t="n"/>
-      <c r="E32" s="20" t="n"/>
-      <c r="F32" s="20" t="n"/>
+      <c r="D32" s="58" t="n"/>
+      <c r="E32" s="58" t="n"/>
+      <c r="F32" s="58" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
@@ -3054,14 +3052,14 @@
         </is>
       </c>
       <c r="B33" s="19" t="n"/>
-      <c r="C33" s="20" t="inlineStr">
+      <c r="C33" s="58" t="inlineStr">
         <is>
           <t>Banquet</t>
         </is>
       </c>
-      <c r="D33" s="20" t="n"/>
-      <c r="E33" s="20" t="n"/>
-      <c r="F33" s="20" t="inlineStr">
+      <c r="D33" s="58" t="n"/>
+      <c r="E33" s="58" t="n"/>
+      <c r="F33" s="58" t="inlineStr">
         <is>
           <t>By invitation only</t>
         </is>
@@ -3145,7 +3143,7 @@
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="51" t="inlineStr">
         <is>
           <t>Keynote 4</t>
         </is>
@@ -3155,12 +3153,12 @@
           <t>Chair: Katsuki Fujisawa</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="51" t="inlineStr">
         <is>
           <t>Mitsuhisa Sato, RIKEN Center for Computational Science</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="51" t="inlineStr">
         <is>
           <t>JHPC Quantum Platform and Applications for Utility-Scale Quantum–HPC Hybrid Computing</t>
         </is>
@@ -3193,14 +3191,14 @@
         </is>
       </c>
       <c r="B5" s="19" t="n"/>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="C5" s="58" t="inlineStr">
         <is>
           <t>Tea Break</t>
         </is>
       </c>
-      <c r="D5" s="20" t="n"/>
-      <c r="E5" s="20" t="n"/>
-      <c r="F5" s="20" t="n"/>
+      <c r="D5" s="58" t="n"/>
+      <c r="E5" s="58" t="n"/>
+      <c r="F5" s="58" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
@@ -3213,22 +3211,22 @@
           <t>SR12</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="55" t="inlineStr">
         <is>
           <t>Quantum Computing for Engineering</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="55" t="inlineStr">
         <is>
           <t>Philippe Codognet &amp; Francisco Chinesta</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="55" t="inlineStr">
         <is>
           <t>Antonio Falco</t>
         </is>
       </c>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="F6" s="55" t="inlineStr">
         <is>
           <t>Encoding Complexity in Quantum Amplitude Estimation for Engineering Numerical Integration</t>
         </is>
@@ -3257,14 +3255,14 @@
     <row r="7">
       <c r="A7" s="17" t="n"/>
       <c r="B7" s="19" t="n"/>
-      <c r="C7" s="20" t="n"/>
-      <c r="D7" s="20" t="n"/>
-      <c r="E7" s="20" t="inlineStr">
+      <c r="C7" s="58" t="n"/>
+      <c r="D7" s="58" t="n"/>
+      <c r="E7" s="58" t="inlineStr">
         <is>
           <t>Kenjiro Terada</t>
         </is>
       </c>
-      <c r="F7" s="20" t="inlineStr">
+      <c r="F7" s="58" t="inlineStr">
         <is>
           <t>Quantum Algorithm for Structural Vibration Analysis</t>
         </is>
@@ -3273,14 +3271,14 @@
     <row r="8">
       <c r="A8" s="17" t="n"/>
       <c r="B8" s="19" t="n"/>
-      <c r="C8" s="20" t="n"/>
-      <c r="D8" s="20" t="n"/>
-      <c r="E8" s="20" t="inlineStr">
+      <c r="C8" s="58" t="n"/>
+      <c r="D8" s="58" t="n"/>
+      <c r="E8" s="58" t="inlineStr">
         <is>
           <t>Frédéric Barbaresco</t>
         </is>
       </c>
-      <c r="F8" s="20" t="inlineStr">
+      <c r="F8" s="58" t="inlineStr">
         <is>
           <t>Quantum Computing for Radar Engineering</t>
         </is>
@@ -3289,14 +3287,14 @@
     <row r="9">
       <c r="A9" s="17" t="n"/>
       <c r="B9" s="19" t="n"/>
-      <c r="C9" s="20" t="n"/>
-      <c r="D9" s="20" t="n"/>
-      <c r="E9" s="20" t="inlineStr">
+      <c r="C9" s="58" t="n"/>
+      <c r="D9" s="58" t="n"/>
+      <c r="E9" s="58" t="inlineStr">
         <is>
           <t>Eloi Gravot</t>
         </is>
       </c>
-      <c r="F9" s="20" t="inlineStr">
+      <c r="F9" s="58" t="inlineStr">
         <is>
           <t>Quantum Annealing for Optimal Monitoring Placement on Transmission Grids</t>
         </is>
@@ -3313,22 +3311,22 @@
           <t>SR1</t>
         </is>
       </c>
-      <c r="C10" s="15" t="inlineStr">
+      <c r="C10" s="55" t="inlineStr">
         <is>
           <t>AI &amp; Data-Driven Methods for Quantitative Finance</t>
         </is>
       </c>
-      <c r="D10" s="15" t="inlineStr">
+      <c r="D10" s="55" t="inlineStr">
         <is>
           <t>Qinxin Yan</t>
         </is>
       </c>
-      <c r="E10" s="15" t="inlineStr">
+      <c r="E10" s="55" t="inlineStr">
         <is>
           <t>Nan Chen</t>
         </is>
       </c>
-      <c r="F10" s="15" t="inlineStr">
+      <c r="F10" s="55" t="inlineStr">
         <is>
           <t>Belief-Augmented Two-Timescale Learning (BATTLE) Algorithm in General-Sum Stochastic Games: Convergence, Equilibrium Selection, and Algorithmic Collusion</t>
         </is>
@@ -3357,14 +3355,14 @@
     <row r="11">
       <c r="A11" s="17" t="n"/>
       <c r="B11" s="19" t="n"/>
-      <c r="C11" s="20" t="n"/>
-      <c r="D11" s="20" t="n"/>
-      <c r="E11" s="20" t="inlineStr">
+      <c r="C11" s="58" t="n"/>
+      <c r="D11" s="58" t="n"/>
+      <c r="E11" s="58" t="inlineStr">
         <is>
           <t>Binnan Wang</t>
         </is>
       </c>
-      <c r="F11" s="20" t="inlineStr">
+      <c r="F11" s="58" t="inlineStr">
         <is>
           <t>Tradable Itô Signatures: A Model-Free, Interpretable Framework for Dynamic Hedging</t>
         </is>
@@ -3373,14 +3371,14 @@
     <row r="12">
       <c r="A12" s="17" t="n"/>
       <c r="B12" s="19" t="n"/>
-      <c r="C12" s="20" t="n"/>
-      <c r="D12" s="20" t="n"/>
-      <c r="E12" s="20" t="inlineStr">
+      <c r="C12" s="58" t="n"/>
+      <c r="D12" s="58" t="n"/>
+      <c r="E12" s="58" t="inlineStr">
         <is>
           <t>Xiang Yu</t>
         </is>
       </c>
-      <c r="F12" s="20" t="inlineStr">
+      <c r="F12" s="58" t="inlineStr">
         <is>
           <t>Deterministic Policy Gradient for Learning Equilibrium in Time-Inconsistent Control Problems</t>
         </is>
@@ -3389,14 +3387,14 @@
     <row r="13">
       <c r="A13" s="17" t="n"/>
       <c r="B13" s="19" t="n"/>
-      <c r="C13" s="20" t="n"/>
-      <c r="D13" s="20" t="n"/>
-      <c r="E13" s="20" t="inlineStr">
+      <c r="C13" s="58" t="n"/>
+      <c r="D13" s="58" t="n"/>
+      <c r="E13" s="58" t="inlineStr">
         <is>
           <t>Qinxin Yan</t>
         </is>
       </c>
-      <c r="F13" s="20" t="inlineStr">
+      <c r="F13" s="58" t="inlineStr">
         <is>
           <t>Sparse Index Tracking with Portfolio Compression and Path Signatures</t>
         </is>
@@ -3413,22 +3411,22 @@
           <t>SR2</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="C14" s="55" t="inlineStr">
         <is>
           <t>Theoretical &amp; Algorithmic Frontiers in Hybrid Quantum–AI Systems</t>
         </is>
       </c>
-      <c r="D14" s="15" t="inlineStr">
+      <c r="D14" s="55" t="inlineStr">
         <is>
           <t>Hongrui Zhang</t>
         </is>
       </c>
-      <c r="E14" s="15" t="inlineStr">
+      <c r="E14" s="55" t="inlineStr">
         <is>
           <t>Hongrui Zhang</t>
         </is>
       </c>
-      <c r="F14" s="15" t="inlineStr">
+      <c r="F14" s="55" t="inlineStr">
         <is>
           <t>Q-Edge: Symmetry-Reduced Quantum Simulation of
 Structured Extreme Dependence</t>
@@ -3458,9 +3456,9 @@
     <row r="15">
       <c r="A15" s="17" t="n"/>
       <c r="B15" s="19" t="n"/>
-      <c r="C15" s="20" t="n"/>
-      <c r="D15" s="20" t="n"/>
-      <c r="E15" s="20" t="inlineStr">
+      <c r="C15" s="58" t="n"/>
+      <c r="D15" s="58" t="n"/>
+      <c r="E15" s="58" t="inlineStr">
         <is>
           <t>Jayne Thompson</t>
         </is>
@@ -3474,9 +3472,9 @@
     <row r="16">
       <c r="A16" s="17" t="n"/>
       <c r="B16" s="19" t="n"/>
-      <c r="C16" s="20" t="n"/>
-      <c r="D16" s="20" t="n"/>
-      <c r="E16" s="20" t="inlineStr">
+      <c r="C16" s="58" t="n"/>
+      <c r="D16" s="58" t="n"/>
+      <c r="E16" s="58" t="inlineStr">
         <is>
           <t>Paul Gregory</t>
         </is>
@@ -3490,8 +3488,8 @@
     <row r="17">
       <c r="A17" s="17" t="n"/>
       <c r="B17" s="19" t="n"/>
-      <c r="C17" s="20" t="n"/>
-      <c r="D17" s="20" t="n"/>
+      <c r="C17" s="58" t="n"/>
+      <c r="D17" s="58" t="n"/>
       <c r="F17" s="22" t="n"/>
     </row>
     <row r="18">
@@ -3505,22 +3503,22 @@
           <t>SR3</t>
         </is>
       </c>
-      <c r="C18" s="15" t="inlineStr">
+      <c r="C18" s="55" t="inlineStr">
         <is>
           <t>Logistics</t>
         </is>
       </c>
-      <c r="D18" s="15" t="inlineStr">
+      <c r="D18" s="55" t="inlineStr">
         <is>
           <t>Ralf Borndörfer</t>
         </is>
       </c>
-      <c r="E18" s="15" t="inlineStr">
+      <c r="E18" s="55" t="inlineStr">
         <is>
           <t>Ralf Borndörfer</t>
         </is>
       </c>
-      <c r="F18" s="15" t="inlineStr">
+      <c r="F18" s="55" t="inlineStr">
         <is>
           <t>Predictive Resource Allocation of Aircraft and Trains</t>
         </is>
@@ -3549,14 +3547,14 @@
     <row r="19">
       <c r="A19" s="17" t="n"/>
       <c r="B19" s="19" t="n"/>
-      <c r="C19" s="20" t="n"/>
-      <c r="D19" s="20" t="n"/>
-      <c r="E19" s="20" t="inlineStr">
+      <c r="C19" s="58" t="n"/>
+      <c r="D19" s="58" t="n"/>
+      <c r="E19" s="58" t="inlineStr">
         <is>
           <t>Boris Grimm</t>
         </is>
       </c>
-      <c r="F19" s="20" t="inlineStr">
+      <c r="F19" s="58" t="inlineStr">
         <is>
           <t>Passenger-Based Intermodal Connection Optimization with Elastic Demands</t>
         </is>
@@ -3565,8 +3563,8 @@
     <row r="20">
       <c r="A20" s="17" t="n"/>
       <c r="B20" s="19" t="n"/>
-      <c r="C20" s="20" t="n"/>
-      <c r="D20" s="20" t="n"/>
+      <c r="C20" s="58" t="n"/>
+      <c r="D20" s="58" t="n"/>
       <c r="E20" s="32" t="inlineStr">
         <is>
           <t>Peng Liu</t>
@@ -3581,14 +3579,14 @@
     <row r="21">
       <c r="A21" s="17" t="n"/>
       <c r="B21" s="19" t="n"/>
-      <c r="C21" s="20" t="n"/>
-      <c r="D21" s="20" t="n"/>
-      <c r="E21" s="20" t="inlineStr">
+      <c r="C21" s="58" t="n"/>
+      <c r="D21" s="58" t="n"/>
+      <c r="E21" s="58" t="inlineStr">
         <is>
           <t>Annika Buchholz</t>
         </is>
       </c>
-      <c r="F21" s="20" t="inlineStr">
+      <c r="F21" s="58" t="inlineStr">
         <is>
           <t>Risk-Aware Unit Commitment: Coupling Bayesian Demand Forecasts with Chance-Constrained and CVaR Optimization</t>
         </is>
@@ -3621,18 +3619,18 @@
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C24" s="24" t="inlineStr">
+      <c r="C24" s="40" t="inlineStr">
         <is>
           <t>Showcase 4</t>
         </is>
       </c>
-      <c r="D24" s="24" t="n"/>
-      <c r="E24" s="24" t="inlineStr">
+      <c r="D24" s="40" t="n"/>
+      <c r="E24" s="40" t="inlineStr">
         <is>
           <t>Dr Hsiao-ju (Rita) Cheng, Future Health Technologies, Singapore-ETH Centre</t>
         </is>
       </c>
-      <c r="F24" s="24" t="inlineStr">
+      <c r="F24" s="40" t="inlineStr">
         <is>
           <t>From Sensor Streams to Therapy Decisions: The AI Opportunity in Post-Stroke Recovery</t>
         </is>
@@ -3669,22 +3667,22 @@
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C25" s="37" t="inlineStr">
+      <c r="C25" s="44" t="inlineStr">
         <is>
           <t>Panel 4: Research, Education, and Talent for the Intelligence Era</t>
         </is>
       </c>
-      <c r="D25" s="37" t="inlineStr">
+      <c r="D25" s="44" t="inlineStr">
         <is>
           <t>Moderator: Ying Chen</t>
         </is>
       </c>
-      <c r="E25" s="37" t="inlineStr">
+      <c r="E25" s="44" t="inlineStr">
         <is>
           <t>Andy Choi, IMDA; Xin Guo, UC Berkeley; José Ignacio Latorre, CQT</t>
         </is>
       </c>
-      <c r="F25" s="37" t="n"/>
+      <c r="F25" s="44" t="n"/>
       <c r="G25" s="39" t="n"/>
       <c r="H25" s="39" t="n"/>
       <c r="I25" s="39" t="n"/>
@@ -3717,14 +3715,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="C26" s="20" t="inlineStr">
+      <c r="C26" s="58" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="D26" s="20" t="n"/>
-      <c r="E26" s="20" t="n"/>
-      <c r="F26" s="20" t="n"/>
+      <c r="D26" s="58" t="n"/>
+      <c r="E26" s="58" t="n"/>
+      <c r="F26" s="58" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
@@ -3737,22 +3735,22 @@
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C27" s="15" t="inlineStr">
+      <c r="C27" s="55" t="inlineStr">
         <is>
           <t>AI for Energy and Finance</t>
         </is>
       </c>
-      <c r="D27" s="15" t="inlineStr">
+      <c r="D27" s="55" t="inlineStr">
         <is>
           <t>Stefan Lessmann</t>
         </is>
       </c>
-      <c r="E27" s="15" t="inlineStr">
+      <c r="E27" s="55" t="inlineStr">
         <is>
           <t>Daniel Traian Pele</t>
         </is>
       </c>
-      <c r="F27" s="15" t="inlineStr">
+      <c r="F27" s="55" t="inlineStr">
         <is>
           <t>One Shift, Two Roles: Diagnosing and Recalibrating Tail Risk Forecasts</t>
         </is>
@@ -3781,14 +3779,14 @@
     <row r="28">
       <c r="A28" s="17" t="n"/>
       <c r="B28" s="19" t="n"/>
-      <c r="C28" s="20" t="n"/>
-      <c r="D28" s="20" t="n"/>
-      <c r="E28" s="20" t="inlineStr">
+      <c r="C28" s="58" t="n"/>
+      <c r="D28" s="58" t="n"/>
+      <c r="E28" s="58" t="inlineStr">
         <is>
           <t>Hoa Thi Nguyen</t>
         </is>
       </c>
-      <c r="F28" s="20" t="inlineStr">
+      <c r="F28" s="58" t="inlineStr">
         <is>
           <t>Robustness in Sequential Decision Making under Evolving Uncertainty: Evidence from High-Frequency Market Making</t>
         </is>
@@ -3797,14 +3795,14 @@
     <row r="29">
       <c r="A29" s="17" t="n"/>
       <c r="B29" s="19" t="n"/>
-      <c r="C29" s="20" t="n"/>
-      <c r="D29" s="20" t="n"/>
-      <c r="E29" s="20" t="inlineStr">
+      <c r="C29" s="58" t="n"/>
+      <c r="D29" s="58" t="n"/>
+      <c r="E29" s="58" t="inlineStr">
         <is>
           <t>Vincent Gurgul</t>
         </is>
       </c>
-      <c r="F29" s="20" t="inlineStr">
+      <c r="F29" s="58" t="inlineStr">
         <is>
           <t>Multi-Objective Divergent Reinforcement Learning for Climate-Conscious Asset Allocation</t>
         </is>
@@ -3813,14 +3811,14 @@
     <row r="30">
       <c r="A30" s="17" t="n"/>
       <c r="B30" s="19" t="n"/>
-      <c r="C30" s="20" t="n"/>
-      <c r="D30" s="20" t="n"/>
-      <c r="E30" s="20" t="inlineStr">
+      <c r="C30" s="58" t="n"/>
+      <c r="D30" s="58" t="n"/>
+      <c r="E30" s="58" t="inlineStr">
         <is>
           <t>Stefan Lessmann</t>
         </is>
       </c>
-      <c r="F30" s="20" t="inlineStr">
+      <c r="F30" s="58" t="inlineStr">
         <is>
           <t>Tabular Foundation Models for Credit Risk Prediction: A Dedicated Review and Empirical Comparison</t>
         </is>
@@ -3837,22 +3835,22 @@
           <t>SR12</t>
         </is>
       </c>
-      <c r="C31" s="15" t="inlineStr">
+      <c r="C31" s="55" t="inlineStr">
         <is>
           <t>Statistics for the AI Era: Reliable Prediction, Responsible Decisions, and Human-Centered Applications</t>
         </is>
       </c>
-      <c r="D31" s="15" t="inlineStr">
+      <c r="D31" s="55" t="inlineStr">
         <is>
           <t>Paulo Canas Rodrigues</t>
         </is>
       </c>
-      <c r="E31" s="15" t="inlineStr">
+      <c r="E31" s="55" t="inlineStr">
         <is>
           <t>Paulo Canas Rodrigues</t>
         </is>
       </c>
-      <c r="F31" s="15" t="inlineStr">
+      <c r="F31" s="55" t="inlineStr">
         <is>
           <t>Why AI Still Needs Statistics: Inference, Uncertainty, and Trust in Modern Learning Systems</t>
         </is>
@@ -3881,14 +3879,14 @@
     <row r="32">
       <c r="A32" s="17" t="n"/>
       <c r="B32" s="19" t="n"/>
-      <c r="C32" s="20" t="n"/>
-      <c r="D32" s="20" t="n"/>
-      <c r="E32" s="20" t="inlineStr">
+      <c r="C32" s="58" t="n"/>
+      <c r="D32" s="58" t="n"/>
+      <c r="E32" s="58" t="inlineStr">
         <is>
           <t>Dedy Dwi Prastyo</t>
         </is>
       </c>
-      <c r="F32" s="20" t="inlineStr">
+      <c r="F32" s="58" t="inlineStr">
         <is>
           <t>Modified LASSO-Based ERNN with MIDAS for Mixed-Frequency Time Series Forecasting</t>
         </is>
@@ -3897,14 +3895,14 @@
     <row r="33">
       <c r="A33" s="17" t="n"/>
       <c r="B33" s="19" t="n"/>
-      <c r="C33" s="20" t="n"/>
-      <c r="D33" s="20" t="n"/>
-      <c r="E33" s="20" t="inlineStr">
+      <c r="C33" s="58" t="n"/>
+      <c r="D33" s="58" t="n"/>
+      <c r="E33" s="58" t="inlineStr">
         <is>
           <t>Jayrold P. Arcede</t>
         </is>
       </c>
-      <c r="F33" s="20" t="inlineStr">
+      <c r="F33" s="58" t="inlineStr">
         <is>
           <t>When AUC Misleads: Constraint Design and Loss-Level Imbalance Correction in Physics-Informed Rare-Event Prediction</t>
         </is>
@@ -3913,14 +3911,14 @@
     <row r="34">
       <c r="A34" s="17" t="n"/>
       <c r="B34" s="19" t="n"/>
-      <c r="C34" s="20" t="n"/>
-      <c r="D34" s="20" t="n"/>
-      <c r="E34" s="20" t="inlineStr">
+      <c r="C34" s="58" t="n"/>
+      <c r="D34" s="58" t="n"/>
+      <c r="E34" s="58" t="inlineStr">
         <is>
           <t>Merliza F. Libao</t>
         </is>
       </c>
-      <c r="F34" s="20" t="inlineStr">
+      <c r="F34" s="58" t="inlineStr">
         <is>
           <t>An Interdisciplinary Human–AI Collaborative Decision Framework for Responsible Human-AI Collaborative Decision Making</t>
         </is>
@@ -3937,22 +3935,22 @@
           <t>SR1</t>
         </is>
       </c>
-      <c r="C35" s="15" t="inlineStr">
+      <c r="C35" s="55" t="inlineStr">
         <is>
           <t>Reinforcement Learning, Security &amp; Autonomous Decision-Making</t>
         </is>
       </c>
-      <c r="D35" s="15" t="inlineStr">
+      <c r="D35" s="55" t="inlineStr">
         <is>
           <t>Lei Zhou</t>
         </is>
       </c>
-      <c r="E35" s="15" t="inlineStr">
+      <c r="E35" s="55" t="inlineStr">
         <is>
           <t>Anand Singh</t>
         </is>
       </c>
-      <c r="F35" s="15" t="inlineStr">
+      <c r="F35" s="55" t="inlineStr">
         <is>
           <t>Reward-Agnostic Stealthy Attacks on Reinforcement Learning via KL-Constrained Adversarial Policies</t>
         </is>
@@ -3981,14 +3979,14 @@
     <row r="36">
       <c r="A36" s="17" t="n"/>
       <c r="B36" s="19" t="n"/>
-      <c r="C36" s="20" t="n"/>
-      <c r="D36" s="20" t="n"/>
-      <c r="E36" s="20" t="inlineStr">
+      <c r="C36" s="58" t="n"/>
+      <c r="D36" s="58" t="n"/>
+      <c r="E36" s="58" t="inlineStr">
         <is>
           <t>Lei Zhou</t>
         </is>
       </c>
-      <c r="F36" s="20" t="inlineStr">
+      <c r="F36" s="58" t="inlineStr">
         <is>
           <t>Learning Optimal Call Policies for Corporate Bonds via Reinforcement Learning</t>
         </is>
@@ -3997,14 +3995,14 @@
     <row r="37">
       <c r="A37" s="17" t="n"/>
       <c r="B37" s="19" t="n"/>
-      <c r="C37" s="20" t="n"/>
-      <c r="D37" s="20" t="n"/>
-      <c r="E37" s="20" t="inlineStr">
+      <c r="C37" s="58" t="n"/>
+      <c r="D37" s="58" t="n"/>
+      <c r="E37" s="58" t="inlineStr">
         <is>
           <t>Naoshi Mihoichi</t>
         </is>
       </c>
-      <c r="F37" s="20" t="inlineStr">
+      <c r="F37" s="58" t="inlineStr">
         <is>
           <t>Vehicle Distance Estimation in Non-Line-of-Sight Scenarios</t>
         </is>
@@ -4013,8 +4011,8 @@
     <row r="38">
       <c r="A38" s="17" t="n"/>
       <c r="B38" s="19" t="n"/>
-      <c r="C38" s="20" t="n"/>
-      <c r="D38" s="20" t="n"/>
+      <c r="C38" s="58" t="n"/>
+      <c r="D38" s="58" t="n"/>
       <c r="E38" s="32" t="inlineStr">
         <is>
           <t>Barbara Tarantino</t>
@@ -4037,22 +4035,22 @@
           <t>SR2</t>
         </is>
       </c>
-      <c r="C39" s="15" t="inlineStr">
+      <c r="C39" s="55" t="inlineStr">
         <is>
           <t>Data Science, AI &amp; Official Statistics</t>
         </is>
       </c>
-      <c r="D39" s="15" t="inlineStr">
+      <c r="D39" s="55" t="inlineStr">
         <is>
           <t>Osuolale Popoola</t>
         </is>
       </c>
-      <c r="E39" s="15" t="inlineStr">
+      <c r="E39" s="55" t="inlineStr">
         <is>
           <t>Osuolale Peter Popoola</t>
         </is>
       </c>
-      <c r="F39" s="15" t="inlineStr">
+      <c r="F39" s="55" t="inlineStr">
         <is>
           <t>The New Data Eco-System and Official Statistics – The General Overview</t>
         </is>
@@ -4081,14 +4079,14 @@
     <row r="40">
       <c r="A40" s="17" t="n"/>
       <c r="B40" s="19" t="n"/>
-      <c r="C40" s="20" t="n"/>
-      <c r="D40" s="20" t="n"/>
-      <c r="E40" s="20" t="inlineStr">
+      <c r="C40" s="58" t="n"/>
+      <c r="D40" s="58" t="n"/>
+      <c r="E40" s="58" t="inlineStr">
         <is>
           <t>Diana Dilshanie Deepawansa</t>
         </is>
       </c>
-      <c r="F40" s="20" t="inlineStr">
+      <c r="F40" s="58" t="inlineStr">
         <is>
           <t>Integrating Data Science and AI Culture for Official Statistics</t>
         </is>
@@ -4097,14 +4095,14 @@
     <row r="41">
       <c r="A41" s="17" t="n"/>
       <c r="B41" s="19" t="n"/>
-      <c r="C41" s="20" t="n"/>
-      <c r="D41" s="20" t="n"/>
-      <c r="E41" s="20" t="inlineStr">
+      <c r="C41" s="58" t="n"/>
+      <c r="D41" s="58" t="n"/>
+      <c r="E41" s="58" t="inlineStr">
         <is>
           <t>Elisabetta Carfagna</t>
         </is>
       </c>
-      <c r="F41" s="20" t="inlineStr">
+      <c r="F41" s="58" t="inlineStr">
         <is>
           <t>Effective Strategies and Skills for AI in Official Statistics</t>
         </is>
@@ -4113,8 +4111,8 @@
     <row r="42">
       <c r="A42" s="17" t="n"/>
       <c r="B42" s="19" t="n"/>
-      <c r="C42" s="20" t="n"/>
-      <c r="D42" s="20" t="n"/>
+      <c r="C42" s="58" t="n"/>
+      <c r="D42" s="58" t="n"/>
       <c r="E42" s="32" t="inlineStr">
         <is>
           <t>Lukas Voss</t>
@@ -4137,22 +4135,22 @@
           <t>SR3</t>
         </is>
       </c>
-      <c r="C43" s="15" t="inlineStr">
+      <c r="C43" s="55" t="inlineStr">
         <is>
           <t>AI for Healthcare</t>
         </is>
       </c>
-      <c r="D43" s="15" t="inlineStr">
+      <c r="D43" s="55" t="inlineStr">
         <is>
           <t>Guan Wang</t>
         </is>
       </c>
-      <c r="E43" s="15" t="inlineStr">
+      <c r="E43" s="55" t="inlineStr">
         <is>
           <t>Xin Guo</t>
         </is>
       </c>
-      <c r="F43" s="15" t="inlineStr">
+      <c r="F43" s="55" t="inlineStr">
         <is>
           <t>Machine Learning for Early Cancer Detection via DNA Methylation</t>
         </is>
@@ -4181,14 +4179,14 @@
     <row r="44">
       <c r="A44" s="17" t="n"/>
       <c r="B44" s="19" t="n"/>
-      <c r="C44" s="20" t="n"/>
-      <c r="D44" s="20" t="n"/>
-      <c r="E44" s="20" t="inlineStr">
+      <c r="C44" s="58" t="n"/>
+      <c r="D44" s="58" t="n"/>
+      <c r="E44" s="58" t="inlineStr">
         <is>
           <t>Guan Wang</t>
         </is>
       </c>
-      <c r="F44" s="20" t="inlineStr">
+      <c r="F44" s="58" t="inlineStr">
         <is>
           <t>Meta-RSI: An Agentic AI Framework for Healthcare</t>
         </is>
@@ -4197,14 +4195,14 @@
     <row r="45">
       <c r="A45" s="17" t="n"/>
       <c r="B45" s="19" t="n"/>
-      <c r="C45" s="20" t="n"/>
-      <c r="D45" s="20" t="n"/>
-      <c r="E45" s="20" t="inlineStr">
+      <c r="C45" s="58" t="n"/>
+      <c r="D45" s="58" t="n"/>
+      <c r="E45" s="58" t="inlineStr">
         <is>
           <t>Yongqi Zhou</t>
         </is>
       </c>
-      <c r="F45" s="20" t="inlineStr">
+      <c r="F45" s="58" t="inlineStr">
         <is>
           <t>Safe Continuous-Time Reinforcement Learning under Limited Interactions</t>
         </is>
@@ -4213,14 +4211,14 @@
     <row r="46">
       <c r="A46" s="17" t="n"/>
       <c r="B46" s="19" t="n"/>
-      <c r="C46" s="20" t="n"/>
-      <c r="D46" s="20" t="n"/>
-      <c r="E46" s="20" t="inlineStr">
+      <c r="C46" s="58" t="n"/>
+      <c r="D46" s="58" t="n"/>
+      <c r="E46" s="58" t="inlineStr">
         <is>
           <t>Grace He</t>
         </is>
       </c>
-      <c r="F46" s="20" t="inlineStr">
+      <c r="F46" s="58" t="inlineStr">
         <is>
           <t>Signature Approach for Contextual Bandits with Nonlinear and Path-dependent Rewards</t>
         </is>
@@ -4257,14 +4255,14 @@
         </is>
       </c>
       <c r="B51" s="19" t="n"/>
-      <c r="C51" s="20" t="inlineStr">
+      <c r="C51" s="58" t="inlineStr">
         <is>
           <t>Tea Break</t>
         </is>
       </c>
-      <c r="D51" s="20" t="n"/>
-      <c r="E51" s="20" t="n"/>
-      <c r="F51" s="20" t="n"/>
+      <c r="D51" s="58" t="n"/>
+      <c r="E51" s="58" t="n"/>
+      <c r="F51" s="58" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -4277,22 +4275,22 @@
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="C52" s="51" t="inlineStr">
         <is>
           <t>Keynote 5</t>
         </is>
       </c>
-      <c r="D52" s="18" t="inlineStr">
+      <c r="D52" s="52" t="inlineStr">
         <is>
           <t>Chair: Stefan Lessmann</t>
         </is>
       </c>
-      <c r="E52" s="6" t="inlineStr">
+      <c r="E52" s="51" t="inlineStr">
         <is>
           <t>Xin Guo, UC Berkeley</t>
         </is>
       </c>
-      <c r="F52" s="6" t="inlineStr">
+      <c r="F52" s="51" t="inlineStr">
         <is>
           <t>Signature-based Time Series Statistical Analysis</t>
         </is>
@@ -4329,22 +4327,22 @@
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C53" s="37" t="inlineStr">
+      <c r="C53" s="44" t="inlineStr">
         <is>
           <t>Panel 5: The Future of Quantum × AI</t>
         </is>
       </c>
-      <c r="D53" s="37" t="inlineStr">
+      <c r="D53" s="44" t="inlineStr">
         <is>
           <t>Moderator: Philippe Codognet</t>
         </is>
       </c>
-      <c r="E53" s="37" t="inlineStr">
+      <c r="E53" s="44" t="inlineStr">
         <is>
           <t>Shaukat Ali, Simula Research Laboratory; Tadashi Kadowaki, AIST G-QuAT / DENSO; Hoong Chuin Lau, SMU; Jeremy Woo, D-Wave</t>
         </is>
       </c>
-      <c r="F53" s="37" t="n"/>
+      <c r="F53" s="44" t="n"/>
       <c r="G53" s="29" t="n"/>
       <c r="H53" s="29" t="n"/>
       <c r="I53" s="29" t="n"/>
@@ -4377,28 +4375,28 @@
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C54" s="20" t="inlineStr">
+      <c r="C54" s="58" t="inlineStr">
         <is>
           <t>Closing Ceremony</t>
         </is>
       </c>
-      <c r="D54" s="20" t="n"/>
-      <c r="E54" s="20" t="n"/>
-      <c r="F54" s="20" t="n"/>
+      <c r="D54" s="58" t="n"/>
+      <c r="E54" s="58" t="n"/>
+      <c r="F54" s="58" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="48" t="n">
         <v>0.75</v>
       </c>
       <c r="B55" s="19" t="n"/>
-      <c r="C55" s="20" t="inlineStr">
+      <c r="C55" s="58" t="inlineStr">
         <is>
           <t>End of Day 3</t>
         </is>
       </c>
-      <c r="D55" s="20" t="n"/>
-      <c r="E55" s="20" t="n"/>
-      <c r="F55" s="20" t="n"/>
+      <c r="D55" s="58" t="n"/>
+      <c r="E55" s="58" t="n"/>
+      <c r="F55" s="58" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
risk session: replace Massimiliano Ferrera with Osamu Takahashi (new talk title)
</commit_message>
<xml_diff>
--- a/public/events/Program.xlsx
+++ b/public/events/Program.xlsx
@@ -1042,12 +1042,12 @@
       <c r="D15" s="58" t="n"/>
       <c r="E15" s="58" t="inlineStr">
         <is>
-          <t>Massimiliano Ferrera</t>
+          <t>Osamu Takahashi</t>
         </is>
       </c>
       <c r="F15" s="58" t="inlineStr">
         <is>
-          <t>Quantum Geometric Entropic Optimization</t>
+          <t>A Matrix Pencil Soft Quantum Kernel for Employee-Retention Analytics</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
keynote 1 chair: Stefan Lessmann; Thorsten Koch joins panel 2, Josef Teichmann joins panel 4
</commit_message>
<xml_diff>
--- a/public/events/Program.xlsx
+++ b/public/events/Program.xlsx
@@ -829,7 +829,7 @@
       </c>
       <c r="D10" s="52" t="inlineStr">
         <is>
-          <t>Chair: Ying Chen</t>
+          <t>Chair: Stefan Lessmann</t>
         </is>
       </c>
       <c r="E10" s="51" t="inlineStr">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="E33" s="44" t="inlineStr">
         <is>
-          <t>Mingshi Koh, NRF; Rosa So, A*STAR/NUS; Tai E Shyong, NUHS/PRECISE/NUS; Toh Han Chong, NCCS/Duke-NUS</t>
+          <t>Thorsten Koch, TU Berlin / ZIB; Mingshi Koh, NRF; Rosa So, A*STAR/NUS; Tai E Shyong, NUHS/PRECISE/NUS; Toh Han Chong, NCCS/Duke-NUS</t>
         </is>
       </c>
       <c r="F33" s="44" t="n"/>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="E25" s="44" t="inlineStr">
         <is>
-          <t>Andy Choi, IMDA; Xin Guo, UC Berkeley; Rizwan Hussain, IBM; José Ignacio Latorre, CQT</t>
+          <t>Andy Choi, IMDA; Xin Guo, UC Berkeley; Rizwan Hussain, IBM; José Ignacio Latorre, CQT; Josef Teichmann, ETH Zurich</t>
         </is>
       </c>
       <c r="F25" s="44" t="n"/>

</xml_diff>

<commit_message>
SR3: Ege Yilmaz & Ariel Neufeld talk titles, speaker affiliations; Teichmann photo on panel card
</commit_message>
<xml_diff>
--- a/public/events/Program.xlsx
+++ b/public/events/Program.xlsx
@@ -1306,7 +1306,7 @@
       </c>
       <c r="E26" s="55" t="inlineStr">
         <is>
-          <t>Hoang Vu</t>
+          <t>Hoang Vu (UCSB)</t>
         </is>
       </c>
       <c r="F26" s="55" t="inlineStr">
@@ -1343,12 +1343,12 @@
       <c r="D27" s="58" t="n"/>
       <c r="E27" s="58" t="inlineStr">
         <is>
-          <t>Ege Yilmaz</t>
+          <t>Ege Yilmaz (U Basel)</t>
         </is>
       </c>
       <c r="F27" s="22" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>Operating Regimes for Scalable Quantum Reservoir Learning</t>
         </is>
       </c>
     </row>
@@ -1359,12 +1359,12 @@
       <c r="D28" s="58" t="n"/>
       <c r="E28" s="58" t="inlineStr">
         <is>
-          <t>Ariel Neufeld</t>
+          <t>Ariel Neufeld (NUS)</t>
         </is>
       </c>
       <c r="F28" s="22" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>Quantum Monte Carlo algorithm for option pricing and its complexity analysis</t>
         </is>
       </c>
     </row>
@@ -1375,7 +1375,7 @@
       <c r="D29" s="58" t="n"/>
       <c r="E29" s="58" t="inlineStr">
         <is>
-          <t>Josef Teichmann</t>
+          <t>Josef Teichmann (ETHZ)</t>
         </is>
       </c>
       <c r="F29" s="58" t="inlineStr">

</xml_diff>

<commit_message>
Quantum Computing for Engineering (SR12): add 5th speaker Richard Hua (CNRS@CREATE)
</commit_message>
<xml_diff>
--- a/public/events/Program.xlsx
+++ b/public/events/Program.xlsx
@@ -3076,7 +3076,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z55"/>
+  <dimension ref="A1:Z56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="36.88" customWidth="1" style="63" min="3" max="3"/>
@@ -3301,72 +3301,68 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="E10" s="58" t="inlineStr">
+        <is>
+          <t>Richard Hua (CNRS@CREATE, Singapore)</t>
+        </is>
+      </c>
+      <c r="F10" s="58" t="inlineStr">
+        <is>
+          <t>Multi-drone route planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>11:00–12:30</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>SR1</t>
         </is>
       </c>
-      <c r="C10" s="55" t="inlineStr">
+      <c r="C11" s="55" t="inlineStr">
         <is>
           <t>AI &amp; Data-Driven Methods for Quantitative Finance</t>
         </is>
       </c>
-      <c r="D10" s="55" t="inlineStr">
+      <c r="D11" s="55" t="inlineStr">
         <is>
           <t>Qinxin Yan</t>
         </is>
       </c>
-      <c r="E10" s="55" t="inlineStr">
+      <c r="E11" s="55" t="inlineStr">
         <is>
           <t>Nan Chen</t>
         </is>
       </c>
-      <c r="F10" s="55" t="inlineStr">
+      <c r="F11" s="55" t="inlineStr">
         <is>
           <t>Belief-Augmented Two-Timescale Learning (BATTLE) Algorithm in General-Sum Stochastic Games: Convergence, Equilibrium Selection, and Algorithmic Collusion</t>
         </is>
       </c>
-      <c r="G10" s="60" t="n"/>
-      <c r="H10" s="60" t="n"/>
-      <c r="I10" s="60" t="n"/>
-      <c r="J10" s="60" t="n"/>
-      <c r="K10" s="60" t="n"/>
-      <c r="L10" s="60" t="n"/>
-      <c r="M10" s="60" t="n"/>
-      <c r="N10" s="60" t="n"/>
-      <c r="O10" s="60" t="n"/>
-      <c r="P10" s="60" t="n"/>
-      <c r="Q10" s="60" t="n"/>
-      <c r="R10" s="60" t="n"/>
-      <c r="S10" s="60" t="n"/>
-      <c r="T10" s="60" t="n"/>
-      <c r="U10" s="60" t="n"/>
-      <c r="V10" s="60" t="n"/>
-      <c r="W10" s="60" t="n"/>
-      <c r="X10" s="60" t="n"/>
-      <c r="Y10" s="60" t="n"/>
-      <c r="Z10" s="60" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="17" t="n"/>
-      <c r="B11" s="19" t="n"/>
-      <c r="C11" s="58" t="n"/>
-      <c r="D11" s="58" t="n"/>
-      <c r="E11" s="58" t="inlineStr">
-        <is>
-          <t>Binnan Wang</t>
-        </is>
-      </c>
-      <c r="F11" s="58" t="inlineStr">
-        <is>
-          <t>Tradable Itô Signatures: A Model-Free, Interpretable Framework for Dynamic Hedging</t>
-        </is>
-      </c>
+      <c r="G11" s="60" t="n"/>
+      <c r="H11" s="60" t="n"/>
+      <c r="I11" s="60" t="n"/>
+      <c r="J11" s="60" t="n"/>
+      <c r="K11" s="60" t="n"/>
+      <c r="L11" s="60" t="n"/>
+      <c r="M11" s="60" t="n"/>
+      <c r="N11" s="60" t="n"/>
+      <c r="O11" s="60" t="n"/>
+      <c r="P11" s="60" t="n"/>
+      <c r="Q11" s="60" t="n"/>
+      <c r="R11" s="60" t="n"/>
+      <c r="S11" s="60" t="n"/>
+      <c r="T11" s="60" t="n"/>
+      <c r="U11" s="60" t="n"/>
+      <c r="V11" s="60" t="n"/>
+      <c r="W11" s="60" t="n"/>
+      <c r="X11" s="60" t="n"/>
+      <c r="Y11" s="60" t="n"/>
+      <c r="Z11" s="60" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="17" t="n"/>
@@ -3375,12 +3371,12 @@
       <c r="D12" s="58" t="n"/>
       <c r="E12" s="58" t="inlineStr">
         <is>
-          <t>Xiang Yu</t>
+          <t>Binnan Wang</t>
         </is>
       </c>
       <c r="F12" s="58" t="inlineStr">
         <is>
-          <t>Deterministic Policy Gradient for Learning Equilibrium in Time-Inconsistent Control Problems</t>
+          <t>Tradable Itô Signatures: A Model-Free, Interpretable Framework for Dynamic Hedging</t>
         </is>
       </c>
     </row>
@@ -3391,83 +3387,83 @@
       <c r="D13" s="58" t="n"/>
       <c r="E13" s="58" t="inlineStr">
         <is>
+          <t>Xiang Yu</t>
+        </is>
+      </c>
+      <c r="F13" s="58" t="inlineStr">
+        <is>
+          <t>Deterministic Policy Gradient for Learning Equilibrium in Time-Inconsistent Control Problems</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="n"/>
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="58" t="n"/>
+      <c r="D14" s="58" t="n"/>
+      <c r="E14" s="58" t="inlineStr">
+        <is>
           <t>Qinxin Yan</t>
         </is>
       </c>
-      <c r="F13" s="58" t="inlineStr">
+      <c r="F14" s="58" t="inlineStr">
         <is>
           <t>Sparse Index Tracking with Portfolio Compression and Path Signatures</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>11:00–12:30</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>SR2</t>
         </is>
       </c>
-      <c r="C14" s="55" t="inlineStr">
+      <c r="C15" s="55" t="inlineStr">
         <is>
           <t>Theoretical &amp; Algorithmic Frontiers in Hybrid Quantum–AI Systems</t>
         </is>
       </c>
-      <c r="D14" s="55" t="inlineStr">
+      <c r="D15" s="55" t="inlineStr">
         <is>
           <t>Hongrui Zhang</t>
         </is>
       </c>
-      <c r="E14" s="55" t="inlineStr">
+      <c r="E15" s="55" t="inlineStr">
         <is>
           <t>Hongrui Zhang</t>
         </is>
       </c>
-      <c r="F14" s="55" t="inlineStr">
+      <c r="F15" s="55" t="inlineStr">
         <is>
           <t>Q-Edge: Symmetry-Reduced Quantum Simulation of
 Structured Extreme Dependence</t>
         </is>
       </c>
-      <c r="G14" s="60" t="n"/>
-      <c r="H14" s="60" t="n"/>
-      <c r="I14" s="60" t="n"/>
-      <c r="J14" s="60" t="n"/>
-      <c r="K14" s="60" t="n"/>
-      <c r="L14" s="60" t="n"/>
-      <c r="M14" s="60" t="n"/>
-      <c r="N14" s="60" t="n"/>
-      <c r="O14" s="60" t="n"/>
-      <c r="P14" s="60" t="n"/>
-      <c r="Q14" s="60" t="n"/>
-      <c r="R14" s="60" t="n"/>
-      <c r="S14" s="60" t="n"/>
-      <c r="T14" s="60" t="n"/>
-      <c r="U14" s="60" t="n"/>
-      <c r="V14" s="60" t="n"/>
-      <c r="W14" s="60" t="n"/>
-      <c r="X14" s="60" t="n"/>
-      <c r="Y14" s="60" t="n"/>
-      <c r="Z14" s="60" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="17" t="n"/>
-      <c r="B15" s="19" t="n"/>
-      <c r="C15" s="58" t="n"/>
-      <c r="D15" s="58" t="n"/>
-      <c r="E15" s="58" t="inlineStr">
-        <is>
-          <t>Jayne Thompson</t>
-        </is>
-      </c>
-      <c r="F15" s="30" t="inlineStr">
-        <is>
-          <t>Error mitigation for midcircuit measurement and feedforward</t>
-        </is>
-      </c>
+      <c r="G15" s="60" t="n"/>
+      <c r="H15" s="60" t="n"/>
+      <c r="I15" s="60" t="n"/>
+      <c r="J15" s="60" t="n"/>
+      <c r="K15" s="60" t="n"/>
+      <c r="L15" s="60" t="n"/>
+      <c r="M15" s="60" t="n"/>
+      <c r="N15" s="60" t="n"/>
+      <c r="O15" s="60" t="n"/>
+      <c r="P15" s="60" t="n"/>
+      <c r="Q15" s="60" t="n"/>
+      <c r="R15" s="60" t="n"/>
+      <c r="S15" s="60" t="n"/>
+      <c r="T15" s="60" t="n"/>
+      <c r="U15" s="60" t="n"/>
+      <c r="V15" s="60" t="n"/>
+      <c r="W15" s="60" t="n"/>
+      <c r="X15" s="60" t="n"/>
+      <c r="Y15" s="60" t="n"/>
+      <c r="Z15" s="60" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="17" t="n"/>
@@ -3476,12 +3472,12 @@
       <c r="D16" s="58" t="n"/>
       <c r="E16" s="58" t="inlineStr">
         <is>
-          <t>Paul Gregory</t>
+          <t>Jayne Thompson</t>
         </is>
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Transport supervision of a time-conditioned circuit Born machine</t>
+          <t>Error mitigation for midcircuit measurement and feedforward</t>
         </is>
       </c>
     </row>
@@ -3490,89 +3486,89 @@
       <c r="B17" s="19" t="n"/>
       <c r="C17" s="58" t="n"/>
       <c r="D17" s="58" t="n"/>
-      <c r="F17" s="22" t="n"/>
+      <c r="E17" s="58" t="inlineStr">
+        <is>
+          <t>Paul Gregory</t>
+        </is>
+      </c>
+      <c r="F17" s="30" t="inlineStr">
+        <is>
+          <t>Transport supervision of a time-conditioned circuit Born machine</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="17" t="n"/>
+      <c r="B18" s="19" t="n"/>
+      <c r="C18" s="58" t="n"/>
+      <c r="D18" s="58" t="n"/>
+      <c r="F18" s="22" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>11:00–12:30</t>
         </is>
       </c>
-      <c r="B18" s="14" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>SR3</t>
         </is>
       </c>
-      <c r="C18" s="55" t="inlineStr">
+      <c r="C19" s="55" t="inlineStr">
         <is>
           <t>Logistics</t>
         </is>
       </c>
-      <c r="D18" s="55" t="inlineStr">
+      <c r="D19" s="55" t="inlineStr">
         <is>
           <t>Ralf Borndörfer</t>
         </is>
       </c>
-      <c r="E18" s="55" t="inlineStr">
+      <c r="E19" s="55" t="inlineStr">
         <is>
           <t>Ralf Borndörfer</t>
         </is>
       </c>
-      <c r="F18" s="55" t="inlineStr">
+      <c r="F19" s="55" t="inlineStr">
         <is>
           <t>Predictive Resource Allocation of Aircraft and Trains</t>
         </is>
       </c>
-      <c r="G18" s="60" t="n"/>
-      <c r="H18" s="60" t="n"/>
-      <c r="I18" s="60" t="n"/>
-      <c r="J18" s="60" t="n"/>
-      <c r="K18" s="60" t="n"/>
-      <c r="L18" s="60" t="n"/>
-      <c r="M18" s="60" t="n"/>
-      <c r="N18" s="60" t="n"/>
-      <c r="O18" s="60" t="n"/>
-      <c r="P18" s="60" t="n"/>
-      <c r="Q18" s="60" t="n"/>
-      <c r="R18" s="60" t="n"/>
-      <c r="S18" s="60" t="n"/>
-      <c r="T18" s="60" t="n"/>
-      <c r="U18" s="60" t="n"/>
-      <c r="V18" s="60" t="n"/>
-      <c r="W18" s="60" t="n"/>
-      <c r="X18" s="60" t="n"/>
-      <c r="Y18" s="60" t="n"/>
-      <c r="Z18" s="60" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="17" t="n"/>
-      <c r="B19" s="19" t="n"/>
-      <c r="C19" s="58" t="n"/>
-      <c r="D19" s="58" t="n"/>
-      <c r="E19" s="58" t="inlineStr">
-        <is>
-          <t>Boris Grimm</t>
-        </is>
-      </c>
-      <c r="F19" s="58" t="inlineStr">
-        <is>
-          <t>Passenger-Based Intermodal Connection Optimization with Elastic Demands</t>
-        </is>
-      </c>
+      <c r="G19" s="60" t="n"/>
+      <c r="H19" s="60" t="n"/>
+      <c r="I19" s="60" t="n"/>
+      <c r="J19" s="60" t="n"/>
+      <c r="K19" s="60" t="n"/>
+      <c r="L19" s="60" t="n"/>
+      <c r="M19" s="60" t="n"/>
+      <c r="N19" s="60" t="n"/>
+      <c r="O19" s="60" t="n"/>
+      <c r="P19" s="60" t="n"/>
+      <c r="Q19" s="60" t="n"/>
+      <c r="R19" s="60" t="n"/>
+      <c r="S19" s="60" t="n"/>
+      <c r="T19" s="60" t="n"/>
+      <c r="U19" s="60" t="n"/>
+      <c r="V19" s="60" t="n"/>
+      <c r="W19" s="60" t="n"/>
+      <c r="X19" s="60" t="n"/>
+      <c r="Y19" s="60" t="n"/>
+      <c r="Z19" s="60" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="17" t="n"/>
       <c r="B20" s="19" t="n"/>
       <c r="C20" s="58" t="n"/>
       <c r="D20" s="58" t="n"/>
-      <c r="E20" s="32" t="inlineStr">
-        <is>
-          <t>Peng Liu</t>
-        </is>
-      </c>
-      <c r="F20" s="32" t="inlineStr">
-        <is>
-          <t>Differentiable Scenario Optimization for Multi-Period Portfolio Construction</t>
+      <c r="E20" s="58" t="inlineStr">
+        <is>
+          <t>Boris Grimm</t>
+        </is>
+      </c>
+      <c r="F20" s="58" t="inlineStr">
+        <is>
+          <t>Passenger-Based Intermodal Connection Optimization with Elastic Demands</t>
         </is>
       </c>
     </row>
@@ -3581,216 +3577,216 @@
       <c r="B21" s="19" t="n"/>
       <c r="C21" s="58" t="n"/>
       <c r="D21" s="58" t="n"/>
-      <c r="E21" s="58" t="inlineStr">
+      <c r="E21" s="32" t="inlineStr">
+        <is>
+          <t>Peng Liu</t>
+        </is>
+      </c>
+      <c r="F21" s="32" t="inlineStr">
+        <is>
+          <t>Differentiable Scenario Optimization for Multi-Period Portfolio Construction</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="n"/>
+      <c r="B22" s="19" t="n"/>
+      <c r="C22" s="58" t="n"/>
+      <c r="D22" s="58" t="n"/>
+      <c r="E22" s="58" t="inlineStr">
         <is>
           <t>Annika Buchholz</t>
         </is>
       </c>
-      <c r="F21" s="58" t="inlineStr">
+      <c r="F22" s="58" t="inlineStr">
         <is>
           <t>Risk-Aware Unit Commitment: Coupling Bayesian Demand Forecasts with Chance-Constrained and CVaR Optimization</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="17" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>11:00–12:30</t>
         </is>
       </c>
-      <c r="B22" s="33" t="inlineStr">
+      <c r="B23" s="33" t="inlineStr">
         <is>
           <t>SR4</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="17" t="n"/>
-      <c r="B23" s="19" t="n"/>
-    </row>
     <row r="24">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="A24" s="17" t="n"/>
+      <c r="B24" s="19" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="21" t="inlineStr">
         <is>
           <t>11:00–11:30</t>
         </is>
       </c>
-      <c r="B24" s="21" t="inlineStr">
+      <c r="B25" s="21" t="inlineStr">
         <is>
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C24" s="40" t="inlineStr">
+      <c r="C25" s="40" t="inlineStr">
         <is>
           <t>Showcase 4</t>
         </is>
       </c>
-      <c r="D24" s="40" t="n"/>
-      <c r="E24" s="40" t="inlineStr">
+      <c r="D25" s="40" t="n"/>
+      <c r="E25" s="40" t="inlineStr">
         <is>
           <t>Dr Hsiao-ju (Rita) Cheng, Future Health Technologies, Singapore-ETH Centre</t>
         </is>
       </c>
-      <c r="F24" s="40" t="inlineStr">
+      <c r="F25" s="40" t="inlineStr">
         <is>
           <t>From Sensor Streams to Therapy Decisions: The AI Opportunity in Post-Stroke Recovery</t>
         </is>
       </c>
-      <c r="G24" s="34" t="n"/>
-      <c r="H24" s="34" t="n"/>
-      <c r="I24" s="34" t="n"/>
-      <c r="J24" s="34" t="n"/>
-      <c r="K24" s="34" t="n"/>
-      <c r="L24" s="34" t="n"/>
-      <c r="M24" s="34" t="n"/>
-      <c r="N24" s="34" t="n"/>
-      <c r="O24" s="34" t="n"/>
-      <c r="P24" s="34" t="n"/>
-      <c r="Q24" s="34" t="n"/>
-      <c r="R24" s="34" t="n"/>
-      <c r="S24" s="34" t="n"/>
-      <c r="T24" s="34" t="n"/>
-      <c r="U24" s="34" t="n"/>
-      <c r="V24" s="34" t="n"/>
-      <c r="W24" s="34" t="n"/>
-      <c r="X24" s="34" t="n"/>
-      <c r="Y24" s="34" t="n"/>
-      <c r="Z24" s="34" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="26" t="inlineStr">
+      <c r="G25" s="34" t="n"/>
+      <c r="H25" s="34" t="n"/>
+      <c r="I25" s="34" t="n"/>
+      <c r="J25" s="34" t="n"/>
+      <c r="K25" s="34" t="n"/>
+      <c r="L25" s="34" t="n"/>
+      <c r="M25" s="34" t="n"/>
+      <c r="N25" s="34" t="n"/>
+      <c r="O25" s="34" t="n"/>
+      <c r="P25" s="34" t="n"/>
+      <c r="Q25" s="34" t="n"/>
+      <c r="R25" s="34" t="n"/>
+      <c r="S25" s="34" t="n"/>
+      <c r="T25" s="34" t="n"/>
+      <c r="U25" s="34" t="n"/>
+      <c r="V25" s="34" t="n"/>
+      <c r="W25" s="34" t="n"/>
+      <c r="X25" s="34" t="n"/>
+      <c r="Y25" s="34" t="n"/>
+      <c r="Z25" s="34" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="26" t="inlineStr">
         <is>
           <t>11:30–12:30</t>
         </is>
       </c>
-      <c r="B25" s="26" t="inlineStr">
+      <c r="B26" s="26" t="inlineStr">
         <is>
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C25" s="44" t="inlineStr">
+      <c r="C26" s="44" t="inlineStr">
         <is>
           <t>Panel 4: Research, Education, and Talent for the Intelligence Era</t>
         </is>
       </c>
-      <c r="D25" s="44" t="inlineStr">
+      <c r="D26" s="44" t="inlineStr">
         <is>
           <t>Moderator: Ying Chen</t>
         </is>
       </c>
-      <c r="E25" s="44" t="inlineStr">
+      <c r="E26" s="44" t="inlineStr">
         <is>
           <t>Andy Choi, IMDA; Xin Guo, UC Berkeley; Rizwan Hussain, IBM; José Ignacio Latorre, CQT; Josef Teichmann, ETH Zurich</t>
         </is>
       </c>
-      <c r="F25" s="44" t="n"/>
-      <c r="G25" s="39" t="n"/>
-      <c r="H25" s="39" t="n"/>
-      <c r="I25" s="39" t="n"/>
-      <c r="J25" s="39" t="n"/>
-      <c r="K25" s="39" t="n"/>
-      <c r="L25" s="39" t="n"/>
-      <c r="M25" s="39" t="n"/>
-      <c r="N25" s="39" t="n"/>
-      <c r="O25" s="39" t="n"/>
-      <c r="P25" s="39" t="n"/>
-      <c r="Q25" s="39" t="n"/>
-      <c r="R25" s="39" t="n"/>
-      <c r="S25" s="39" t="n"/>
-      <c r="T25" s="39" t="n"/>
-      <c r="U25" s="39" t="n"/>
-      <c r="V25" s="39" t="n"/>
-      <c r="W25" s="39" t="n"/>
-      <c r="X25" s="39" t="n"/>
-      <c r="Y25" s="39" t="n"/>
-      <c r="Z25" s="39" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="17" t="inlineStr">
+      <c r="F26" s="44" t="n"/>
+      <c r="G26" s="39" t="n"/>
+      <c r="H26" s="39" t="n"/>
+      <c r="I26" s="39" t="n"/>
+      <c r="J26" s="39" t="n"/>
+      <c r="K26" s="39" t="n"/>
+      <c r="L26" s="39" t="n"/>
+      <c r="M26" s="39" t="n"/>
+      <c r="N26" s="39" t="n"/>
+      <c r="O26" s="39" t="n"/>
+      <c r="P26" s="39" t="n"/>
+      <c r="Q26" s="39" t="n"/>
+      <c r="R26" s="39" t="n"/>
+      <c r="S26" s="39" t="n"/>
+      <c r="T26" s="39" t="n"/>
+      <c r="U26" s="39" t="n"/>
+      <c r="V26" s="39" t="n"/>
+      <c r="W26" s="39" t="n"/>
+      <c r="X26" s="39" t="n"/>
+      <c r="Y26" s="39" t="n"/>
+      <c r="Z26" s="39" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>12:30–13:30</t>
         </is>
       </c>
-      <c r="B26" s="19" t="inlineStr">
+      <c r="B27" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C26" s="58" t="inlineStr">
+      <c r="C27" s="58" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="D26" s="58" t="n"/>
-      <c r="E26" s="58" t="n"/>
-      <c r="F26" s="58" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="D27" s="58" t="n"/>
+      <c r="E27" s="58" t="n"/>
+      <c r="F27" s="58" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
         <is>
           <t>13:30–15:00</t>
         </is>
       </c>
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C27" s="55" t="inlineStr">
+      <c r="C28" s="55" t="inlineStr">
         <is>
           <t>AI for Energy and Finance</t>
         </is>
       </c>
-      <c r="D27" s="55" t="inlineStr">
+      <c r="D28" s="55" t="inlineStr">
         <is>
           <t>Stefan Lessmann</t>
         </is>
       </c>
-      <c r="E27" s="55" t="inlineStr">
+      <c r="E28" s="55" t="inlineStr">
         <is>
           <t>Daniel Traian Pele</t>
         </is>
       </c>
-      <c r="F27" s="55" t="inlineStr">
+      <c r="F28" s="55" t="inlineStr">
         <is>
           <t>One Shift, Two Roles: Diagnosing and Recalibrating Tail Risk Forecasts</t>
         </is>
       </c>
-      <c r="G27" s="60" t="n"/>
-      <c r="H27" s="60" t="n"/>
-      <c r="I27" s="60" t="n"/>
-      <c r="J27" s="60" t="n"/>
-      <c r="K27" s="60" t="n"/>
-      <c r="L27" s="60" t="n"/>
-      <c r="M27" s="60" t="n"/>
-      <c r="N27" s="60" t="n"/>
-      <c r="O27" s="60" t="n"/>
-      <c r="P27" s="60" t="n"/>
-      <c r="Q27" s="60" t="n"/>
-      <c r="R27" s="60" t="n"/>
-      <c r="S27" s="60" t="n"/>
-      <c r="T27" s="60" t="n"/>
-      <c r="U27" s="60" t="n"/>
-      <c r="V27" s="60" t="n"/>
-      <c r="W27" s="60" t="n"/>
-      <c r="X27" s="60" t="n"/>
-      <c r="Y27" s="60" t="n"/>
-      <c r="Z27" s="60" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="17" t="n"/>
-      <c r="B28" s="19" t="n"/>
-      <c r="C28" s="58" t="n"/>
-      <c r="D28" s="58" t="n"/>
-      <c r="E28" s="58" t="inlineStr">
-        <is>
-          <t>Hoa Thi Nguyen</t>
-        </is>
-      </c>
-      <c r="F28" s="58" t="inlineStr">
-        <is>
-          <t>Robustness in Sequential Decision Making under Evolving Uncertainty: Evidence from High-Frequency Market Making</t>
-        </is>
-      </c>
+      <c r="G28" s="60" t="n"/>
+      <c r="H28" s="60" t="n"/>
+      <c r="I28" s="60" t="n"/>
+      <c r="J28" s="60" t="n"/>
+      <c r="K28" s="60" t="n"/>
+      <c r="L28" s="60" t="n"/>
+      <c r="M28" s="60" t="n"/>
+      <c r="N28" s="60" t="n"/>
+      <c r="O28" s="60" t="n"/>
+      <c r="P28" s="60" t="n"/>
+      <c r="Q28" s="60" t="n"/>
+      <c r="R28" s="60" t="n"/>
+      <c r="S28" s="60" t="n"/>
+      <c r="T28" s="60" t="n"/>
+      <c r="U28" s="60" t="n"/>
+      <c r="V28" s="60" t="n"/>
+      <c r="W28" s="60" t="n"/>
+      <c r="X28" s="60" t="n"/>
+      <c r="Y28" s="60" t="n"/>
+      <c r="Z28" s="60" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="17" t="n"/>
@@ -3799,12 +3795,12 @@
       <c r="D29" s="58" t="n"/>
       <c r="E29" s="58" t="inlineStr">
         <is>
-          <t>Vincent Gurgul</t>
+          <t>Hoa Thi Nguyen</t>
         </is>
       </c>
       <c r="F29" s="58" t="inlineStr">
         <is>
-          <t>Multi-Objective Divergent Reinforcement Learning for Climate-Conscious Asset Allocation</t>
+          <t>Robustness in Sequential Decision Making under Evolving Uncertainty: Evidence from High-Frequency Market Making</t>
         </is>
       </c>
     </row>
@@ -3815,82 +3811,82 @@
       <c r="D30" s="58" t="n"/>
       <c r="E30" s="58" t="inlineStr">
         <is>
+          <t>Vincent Gurgul</t>
+        </is>
+      </c>
+      <c r="F30" s="58" t="inlineStr">
+        <is>
+          <t>Multi-Objective Divergent Reinforcement Learning for Climate-Conscious Asset Allocation</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="n"/>
+      <c r="B31" s="19" t="n"/>
+      <c r="C31" s="58" t="n"/>
+      <c r="D31" s="58" t="n"/>
+      <c r="E31" s="58" t="inlineStr">
+        <is>
           <t>Stefan Lessmann</t>
         </is>
       </c>
-      <c r="F30" s="58" t="inlineStr">
+      <c r="F31" s="58" t="inlineStr">
         <is>
           <t>Tabular Foundation Models for Credit Risk Prediction: A Dedicated Review and Empirical Comparison</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="13" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
         <is>
           <t>13:30–15:00</t>
         </is>
       </c>
-      <c r="B31" s="14" t="inlineStr">
+      <c r="B32" s="14" t="inlineStr">
         <is>
           <t>SR12</t>
         </is>
       </c>
-      <c r="C31" s="55" t="inlineStr">
+      <c r="C32" s="55" t="inlineStr">
         <is>
           <t>Statistics for the AI Era: Reliable Prediction, Responsible Decisions, and Human-Centered Applications</t>
         </is>
       </c>
-      <c r="D31" s="55" t="inlineStr">
+      <c r="D32" s="55" t="inlineStr">
         <is>
           <t>Paulo Canas Rodrigues</t>
         </is>
       </c>
-      <c r="E31" s="55" t="inlineStr">
+      <c r="E32" s="55" t="inlineStr">
         <is>
           <t>Paulo Canas Rodrigues</t>
         </is>
       </c>
-      <c r="F31" s="55" t="inlineStr">
+      <c r="F32" s="55" t="inlineStr">
         <is>
           <t>Why AI Still Needs Statistics: Inference, Uncertainty, and Trust in Modern Learning Systems</t>
         </is>
       </c>
-      <c r="G31" s="60" t="n"/>
-      <c r="H31" s="60" t="n"/>
-      <c r="I31" s="60" t="n"/>
-      <c r="J31" s="60" t="n"/>
-      <c r="K31" s="60" t="n"/>
-      <c r="L31" s="60" t="n"/>
-      <c r="M31" s="60" t="n"/>
-      <c r="N31" s="60" t="n"/>
-      <c r="O31" s="60" t="n"/>
-      <c r="P31" s="60" t="n"/>
-      <c r="Q31" s="60" t="n"/>
-      <c r="R31" s="60" t="n"/>
-      <c r="S31" s="60" t="n"/>
-      <c r="T31" s="60" t="n"/>
-      <c r="U31" s="60" t="n"/>
-      <c r="V31" s="60" t="n"/>
-      <c r="W31" s="60" t="n"/>
-      <c r="X31" s="60" t="n"/>
-      <c r="Y31" s="60" t="n"/>
-      <c r="Z31" s="60" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="17" t="n"/>
-      <c r="B32" s="19" t="n"/>
-      <c r="C32" s="58" t="n"/>
-      <c r="D32" s="58" t="n"/>
-      <c r="E32" s="58" t="inlineStr">
-        <is>
-          <t>Dedy Dwi Prastyo</t>
-        </is>
-      </c>
-      <c r="F32" s="58" t="inlineStr">
-        <is>
-          <t>Modified LASSO-Based ERNN with MIDAS for Mixed-Frequency Time Series Forecasting</t>
-        </is>
-      </c>
+      <c r="G32" s="60" t="n"/>
+      <c r="H32" s="60" t="n"/>
+      <c r="I32" s="60" t="n"/>
+      <c r="J32" s="60" t="n"/>
+      <c r="K32" s="60" t="n"/>
+      <c r="L32" s="60" t="n"/>
+      <c r="M32" s="60" t="n"/>
+      <c r="N32" s="60" t="n"/>
+      <c r="O32" s="60" t="n"/>
+      <c r="P32" s="60" t="n"/>
+      <c r="Q32" s="60" t="n"/>
+      <c r="R32" s="60" t="n"/>
+      <c r="S32" s="60" t="n"/>
+      <c r="T32" s="60" t="n"/>
+      <c r="U32" s="60" t="n"/>
+      <c r="V32" s="60" t="n"/>
+      <c r="W32" s="60" t="n"/>
+      <c r="X32" s="60" t="n"/>
+      <c r="Y32" s="60" t="n"/>
+      <c r="Z32" s="60" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="17" t="n"/>
@@ -3899,12 +3895,12 @@
       <c r="D33" s="58" t="n"/>
       <c r="E33" s="58" t="inlineStr">
         <is>
-          <t>Jayrold P. Arcede</t>
+          <t>Dedy Dwi Prastyo</t>
         </is>
       </c>
       <c r="F33" s="58" t="inlineStr">
         <is>
-          <t>When AUC Misleads: Constraint Design and Loss-Level Imbalance Correction in Physics-Informed Rare-Event Prediction</t>
+          <t>Modified LASSO-Based ERNN with MIDAS for Mixed-Frequency Time Series Forecasting</t>
         </is>
       </c>
     </row>
@@ -3915,82 +3911,82 @@
       <c r="D34" s="58" t="n"/>
       <c r="E34" s="58" t="inlineStr">
         <is>
+          <t>Jayrold P. Arcede</t>
+        </is>
+      </c>
+      <c r="F34" s="58" t="inlineStr">
+        <is>
+          <t>When AUC Misleads: Constraint Design and Loss-Level Imbalance Correction in Physics-Informed Rare-Event Prediction</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="17" t="n"/>
+      <c r="B35" s="19" t="n"/>
+      <c r="C35" s="58" t="n"/>
+      <c r="D35" s="58" t="n"/>
+      <c r="E35" s="58" t="inlineStr">
+        <is>
           <t>Merliza F. Libao</t>
         </is>
       </c>
-      <c r="F34" s="58" t="inlineStr">
+      <c r="F35" s="58" t="inlineStr">
         <is>
           <t>An Interdisciplinary Human–AI Collaborative Decision Framework for Responsible Human-AI Collaborative Decision Making</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="13" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
         <is>
           <t>13:30–15:00</t>
         </is>
       </c>
-      <c r="B35" s="14" t="inlineStr">
+      <c r="B36" s="14" t="inlineStr">
         <is>
           <t>SR1</t>
         </is>
       </c>
-      <c r="C35" s="55" t="inlineStr">
+      <c r="C36" s="55" t="inlineStr">
         <is>
           <t>Reinforcement Learning, Security &amp; Autonomous Decision-Making</t>
         </is>
       </c>
-      <c r="D35" s="55" t="inlineStr">
+      <c r="D36" s="55" t="inlineStr">
         <is>
           <t>Lei Zhou</t>
         </is>
       </c>
-      <c r="E35" s="55" t="inlineStr">
+      <c r="E36" s="55" t="inlineStr">
         <is>
           <t>Anand Singh</t>
         </is>
       </c>
-      <c r="F35" s="55" t="inlineStr">
+      <c r="F36" s="55" t="inlineStr">
         <is>
           <t>Reward-Agnostic Stealthy Attacks on Reinforcement Learning via KL-Constrained Adversarial Policies</t>
         </is>
       </c>
-      <c r="G35" s="60" t="n"/>
-      <c r="H35" s="60" t="n"/>
-      <c r="I35" s="60" t="n"/>
-      <c r="J35" s="60" t="n"/>
-      <c r="K35" s="60" t="n"/>
-      <c r="L35" s="60" t="n"/>
-      <c r="M35" s="60" t="n"/>
-      <c r="N35" s="60" t="n"/>
-      <c r="O35" s="60" t="n"/>
-      <c r="P35" s="60" t="n"/>
-      <c r="Q35" s="60" t="n"/>
-      <c r="R35" s="60" t="n"/>
-      <c r="S35" s="60" t="n"/>
-      <c r="T35" s="60" t="n"/>
-      <c r="U35" s="60" t="n"/>
-      <c r="V35" s="60" t="n"/>
-      <c r="W35" s="60" t="n"/>
-      <c r="X35" s="60" t="n"/>
-      <c r="Y35" s="60" t="n"/>
-      <c r="Z35" s="60" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="17" t="n"/>
-      <c r="B36" s="19" t="n"/>
-      <c r="C36" s="58" t="n"/>
-      <c r="D36" s="58" t="n"/>
-      <c r="E36" s="58" t="inlineStr">
-        <is>
-          <t>Lei Zhou</t>
-        </is>
-      </c>
-      <c r="F36" s="58" t="inlineStr">
-        <is>
-          <t>Learning Optimal Call Policies for Corporate Bonds via Reinforcement Learning</t>
-        </is>
-      </c>
+      <c r="G36" s="60" t="n"/>
+      <c r="H36" s="60" t="n"/>
+      <c r="I36" s="60" t="n"/>
+      <c r="J36" s="60" t="n"/>
+      <c r="K36" s="60" t="n"/>
+      <c r="L36" s="60" t="n"/>
+      <c r="M36" s="60" t="n"/>
+      <c r="N36" s="60" t="n"/>
+      <c r="O36" s="60" t="n"/>
+      <c r="P36" s="60" t="n"/>
+      <c r="Q36" s="60" t="n"/>
+      <c r="R36" s="60" t="n"/>
+      <c r="S36" s="60" t="n"/>
+      <c r="T36" s="60" t="n"/>
+      <c r="U36" s="60" t="n"/>
+      <c r="V36" s="60" t="n"/>
+      <c r="W36" s="60" t="n"/>
+      <c r="X36" s="60" t="n"/>
+      <c r="Y36" s="60" t="n"/>
+      <c r="Z36" s="60" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="17" t="n"/>
@@ -3999,12 +3995,12 @@
       <c r="D37" s="58" t="n"/>
       <c r="E37" s="58" t="inlineStr">
         <is>
-          <t>Naoshi Mihoichi</t>
+          <t>Lei Zhou</t>
         </is>
       </c>
       <c r="F37" s="58" t="inlineStr">
         <is>
-          <t>Vehicle Distance Estimation in Non-Line-of-Sight Scenarios</t>
+          <t>Learning Optimal Call Policies for Corporate Bonds via Reinforcement Learning</t>
         </is>
       </c>
     </row>
@@ -4013,84 +4009,84 @@
       <c r="B38" s="19" t="n"/>
       <c r="C38" s="58" t="n"/>
       <c r="D38" s="58" t="n"/>
-      <c r="E38" s="32" t="inlineStr">
+      <c r="E38" s="58" t="inlineStr">
+        <is>
+          <t>Naoshi Mihoichi</t>
+        </is>
+      </c>
+      <c r="F38" s="58" t="inlineStr">
+        <is>
+          <t>Vehicle Distance Estimation in Non-Line-of-Sight Scenarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="n"/>
+      <c r="B39" s="19" t="n"/>
+      <c r="C39" s="58" t="n"/>
+      <c r="D39" s="58" t="n"/>
+      <c r="E39" s="32" t="inlineStr">
         <is>
           <t>Barbara Tarantino</t>
         </is>
       </c>
-      <c r="F38" s="32" t="inlineStr">
+      <c r="F39" s="32" t="inlineStr">
         <is>
           <t>Beyond Accuracy: Metrics for High-Dimensional AI Outputs</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="13" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
         <is>
           <t>13:30–15:00</t>
         </is>
       </c>
-      <c r="B39" s="14" t="inlineStr">
+      <c r="B40" s="14" t="inlineStr">
         <is>
           <t>SR2</t>
         </is>
       </c>
-      <c r="C39" s="55" t="inlineStr">
+      <c r="C40" s="55" t="inlineStr">
         <is>
           <t>Data Science, AI &amp; Official Statistics</t>
         </is>
       </c>
-      <c r="D39" s="55" t="inlineStr">
+      <c r="D40" s="55" t="inlineStr">
         <is>
           <t>Osuolale Popoola</t>
         </is>
       </c>
-      <c r="E39" s="55" t="inlineStr">
+      <c r="E40" s="55" t="inlineStr">
         <is>
           <t>Osuolale Peter Popoola</t>
         </is>
       </c>
-      <c r="F39" s="55" t="inlineStr">
+      <c r="F40" s="55" t="inlineStr">
         <is>
           <t>The New Data Eco-System and Official Statistics – The General Overview</t>
         </is>
       </c>
-      <c r="G39" s="60" t="n"/>
-      <c r="H39" s="60" t="n"/>
-      <c r="I39" s="60" t="n"/>
-      <c r="J39" s="60" t="n"/>
-      <c r="K39" s="60" t="n"/>
-      <c r="L39" s="60" t="n"/>
-      <c r="M39" s="60" t="n"/>
-      <c r="N39" s="60" t="n"/>
-      <c r="O39" s="60" t="n"/>
-      <c r="P39" s="60" t="n"/>
-      <c r="Q39" s="60" t="n"/>
-      <c r="R39" s="60" t="n"/>
-      <c r="S39" s="60" t="n"/>
-      <c r="T39" s="60" t="n"/>
-      <c r="U39" s="60" t="n"/>
-      <c r="V39" s="60" t="n"/>
-      <c r="W39" s="60" t="n"/>
-      <c r="X39" s="60" t="n"/>
-      <c r="Y39" s="60" t="n"/>
-      <c r="Z39" s="60" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="17" t="n"/>
-      <c r="B40" s="19" t="n"/>
-      <c r="C40" s="58" t="n"/>
-      <c r="D40" s="58" t="n"/>
-      <c r="E40" s="58" t="inlineStr">
-        <is>
-          <t>Diana Dilshanie Deepawansa</t>
-        </is>
-      </c>
-      <c r="F40" s="58" t="inlineStr">
-        <is>
-          <t>Integrating Data Science and AI Culture for Official Statistics</t>
-        </is>
-      </c>
+      <c r="G40" s="60" t="n"/>
+      <c r="H40" s="60" t="n"/>
+      <c r="I40" s="60" t="n"/>
+      <c r="J40" s="60" t="n"/>
+      <c r="K40" s="60" t="n"/>
+      <c r="L40" s="60" t="n"/>
+      <c r="M40" s="60" t="n"/>
+      <c r="N40" s="60" t="n"/>
+      <c r="O40" s="60" t="n"/>
+      <c r="P40" s="60" t="n"/>
+      <c r="Q40" s="60" t="n"/>
+      <c r="R40" s="60" t="n"/>
+      <c r="S40" s="60" t="n"/>
+      <c r="T40" s="60" t="n"/>
+      <c r="U40" s="60" t="n"/>
+      <c r="V40" s="60" t="n"/>
+      <c r="W40" s="60" t="n"/>
+      <c r="X40" s="60" t="n"/>
+      <c r="Y40" s="60" t="n"/>
+      <c r="Z40" s="60" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="17" t="n"/>
@@ -4099,12 +4095,12 @@
       <c r="D41" s="58" t="n"/>
       <c r="E41" s="58" t="inlineStr">
         <is>
-          <t>Elisabetta Carfagna</t>
+          <t>Diana Dilshanie Deepawansa</t>
         </is>
       </c>
       <c r="F41" s="58" t="inlineStr">
         <is>
-          <t>Effective Strategies and Skills for AI in Official Statistics</t>
+          <t>Integrating Data Science and AI Culture for Official Statistics</t>
         </is>
       </c>
     </row>
@@ -4113,84 +4109,84 @@
       <c r="B42" s="19" t="n"/>
       <c r="C42" s="58" t="n"/>
       <c r="D42" s="58" t="n"/>
-      <c r="E42" s="32" t="inlineStr">
+      <c r="E42" s="58" t="inlineStr">
+        <is>
+          <t>Elisabetta Carfagna</t>
+        </is>
+      </c>
+      <c r="F42" s="58" t="inlineStr">
+        <is>
+          <t>Effective Strategies and Skills for AI in Official Statistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="n"/>
+      <c r="B43" s="19" t="n"/>
+      <c r="C43" s="58" t="n"/>
+      <c r="D43" s="58" t="n"/>
+      <c r="E43" s="32" t="inlineStr">
         <is>
           <t>Lukas Voss</t>
         </is>
       </c>
-      <c r="F42" s="32" t="inlineStr">
+      <c r="F43" s="32" t="inlineStr">
         <is>
           <t>From Forecast Accuracy to Battery Revenue: Zero-Shot Foundation Models for Day-Ahead and Reserve Markets</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="13" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
         <is>
           <t>13:30–15:00</t>
         </is>
       </c>
-      <c r="B43" s="14" t="inlineStr">
+      <c r="B44" s="14" t="inlineStr">
         <is>
           <t>SR3</t>
         </is>
       </c>
-      <c r="C43" s="55" t="inlineStr">
+      <c r="C44" s="55" t="inlineStr">
         <is>
           <t>AI for Healthcare</t>
         </is>
       </c>
-      <c r="D43" s="55" t="inlineStr">
+      <c r="D44" s="55" t="inlineStr">
         <is>
           <t>Guan Wang</t>
         </is>
       </c>
-      <c r="E43" s="55" t="inlineStr">
+      <c r="E44" s="55" t="inlineStr">
         <is>
           <t>Xin Guo</t>
         </is>
       </c>
-      <c r="F43" s="55" t="inlineStr">
+      <c r="F44" s="55" t="inlineStr">
         <is>
           <t>Machine Learning for Early Cancer Detection via DNA Methylation</t>
         </is>
       </c>
-      <c r="G43" s="60" t="n"/>
-      <c r="H43" s="60" t="n"/>
-      <c r="I43" s="60" t="n"/>
-      <c r="J43" s="60" t="n"/>
-      <c r="K43" s="60" t="n"/>
-      <c r="L43" s="60" t="n"/>
-      <c r="M43" s="60" t="n"/>
-      <c r="N43" s="60" t="n"/>
-      <c r="O43" s="60" t="n"/>
-      <c r="P43" s="60" t="n"/>
-      <c r="Q43" s="60" t="n"/>
-      <c r="R43" s="60" t="n"/>
-      <c r="S43" s="60" t="n"/>
-      <c r="T43" s="60" t="n"/>
-      <c r="U43" s="60" t="n"/>
-      <c r="V43" s="60" t="n"/>
-      <c r="W43" s="60" t="n"/>
-      <c r="X43" s="60" t="n"/>
-      <c r="Y43" s="60" t="n"/>
-      <c r="Z43" s="60" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="17" t="n"/>
-      <c r="B44" s="19" t="n"/>
-      <c r="C44" s="58" t="n"/>
-      <c r="D44" s="58" t="n"/>
-      <c r="E44" s="58" t="inlineStr">
-        <is>
-          <t>Guan Wang</t>
-        </is>
-      </c>
-      <c r="F44" s="58" t="inlineStr">
-        <is>
-          <t>Meta-RSI: An Agentic AI Framework for Healthcare</t>
-        </is>
-      </c>
+      <c r="G44" s="60" t="n"/>
+      <c r="H44" s="60" t="n"/>
+      <c r="I44" s="60" t="n"/>
+      <c r="J44" s="60" t="n"/>
+      <c r="K44" s="60" t="n"/>
+      <c r="L44" s="60" t="n"/>
+      <c r="M44" s="60" t="n"/>
+      <c r="N44" s="60" t="n"/>
+      <c r="O44" s="60" t="n"/>
+      <c r="P44" s="60" t="n"/>
+      <c r="Q44" s="60" t="n"/>
+      <c r="R44" s="60" t="n"/>
+      <c r="S44" s="60" t="n"/>
+      <c r="T44" s="60" t="n"/>
+      <c r="U44" s="60" t="n"/>
+      <c r="V44" s="60" t="n"/>
+      <c r="W44" s="60" t="n"/>
+      <c r="X44" s="60" t="n"/>
+      <c r="Y44" s="60" t="n"/>
+      <c r="Z44" s="60" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="17" t="n"/>
@@ -4199,12 +4195,12 @@
       <c r="D45" s="58" t="n"/>
       <c r="E45" s="58" t="inlineStr">
         <is>
-          <t>Yongqi Zhou</t>
+          <t>Guan Wang</t>
         </is>
       </c>
       <c r="F45" s="58" t="inlineStr">
         <is>
-          <t>Safe Continuous-Time Reinforcement Learning under Limited Interactions</t>
+          <t>Meta-RSI: An Agentic AI Framework for Healthcare</t>
         </is>
       </c>
     </row>
@@ -4215,30 +4211,42 @@
       <c r="D46" s="58" t="n"/>
       <c r="E46" s="58" t="inlineStr">
         <is>
+          <t>Yongqi Zhou</t>
+        </is>
+      </c>
+      <c r="F46" s="58" t="inlineStr">
+        <is>
+          <t>Safe Continuous-Time Reinforcement Learning under Limited Interactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="n"/>
+      <c r="B47" s="19" t="n"/>
+      <c r="C47" s="58" t="n"/>
+      <c r="D47" s="58" t="n"/>
+      <c r="E47" s="58" t="inlineStr">
+        <is>
           <t>Grace He</t>
         </is>
       </c>
-      <c r="F46" s="58" t="inlineStr">
+      <c r="F47" s="58" t="inlineStr">
         <is>
           <t>Signature Approach for Contextual Bandits with Nonlinear and Path-dependent Rewards</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="17" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="17" t="inlineStr">
         <is>
           <t>13:30–15:00</t>
         </is>
       </c>
-      <c r="B47" s="33" t="inlineStr">
+      <c r="B48" s="33" t="inlineStr">
         <is>
           <t>SR4</t>
         </is>
       </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="17" t="n"/>
-      <c r="B48" s="19" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="17" t="n"/>
@@ -4249,154 +4257,158 @@
       <c r="B50" s="19" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="17" t="inlineStr">
+      <c r="A51" s="17" t="n"/>
+      <c r="B51" s="19" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
         <is>
           <t>15:00–15:30</t>
         </is>
       </c>
-      <c r="B51" s="19" t="n"/>
-      <c r="C51" s="58" t="inlineStr">
+      <c r="B52" s="19" t="n"/>
+      <c r="C52" s="58" t="inlineStr">
         <is>
           <t>Tea Break</t>
         </is>
       </c>
-      <c r="D51" s="58" t="n"/>
-      <c r="E51" s="58" t="n"/>
-      <c r="F51" s="58" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="3" t="inlineStr">
+      <c r="D52" s="58" t="n"/>
+      <c r="E52" s="58" t="n"/>
+      <c r="F52" s="58" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>15:30–16:30</t>
         </is>
       </c>
-      <c r="B52" s="4" t="inlineStr">
+      <c r="B53" s="4" t="inlineStr">
         <is>
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C52" s="51" t="inlineStr">
+      <c r="C53" s="51" t="inlineStr">
         <is>
           <t>Keynote 5</t>
         </is>
       </c>
-      <c r="D52" s="52" t="inlineStr">
+      <c r="D53" s="52" t="inlineStr">
         <is>
           <t>Chair: Stefan Lessmann</t>
         </is>
       </c>
-      <c r="E52" s="51" t="inlineStr">
+      <c r="E53" s="51" t="inlineStr">
         <is>
           <t>Xin Guo, UC Berkeley</t>
         </is>
       </c>
-      <c r="F52" s="51" t="inlineStr">
+      <c r="F53" s="51" t="inlineStr">
         <is>
           <t>Signature-based Time Series Statistical Analysis</t>
         </is>
       </c>
-      <c r="G52" s="12" t="n"/>
-      <c r="H52" s="12" t="n"/>
-      <c r="I52" s="12" t="n"/>
-      <c r="J52" s="12" t="n"/>
-      <c r="K52" s="12" t="n"/>
-      <c r="L52" s="12" t="n"/>
-      <c r="M52" s="12" t="n"/>
-      <c r="N52" s="12" t="n"/>
-      <c r="O52" s="12" t="n"/>
-      <c r="P52" s="12" t="n"/>
-      <c r="Q52" s="12" t="n"/>
-      <c r="R52" s="12" t="n"/>
-      <c r="S52" s="12" t="n"/>
-      <c r="T52" s="12" t="n"/>
-      <c r="U52" s="12" t="n"/>
-      <c r="V52" s="12" t="n"/>
-      <c r="W52" s="12" t="n"/>
-      <c r="X52" s="12" t="n"/>
-      <c r="Y52" s="12" t="n"/>
-      <c r="Z52" s="12" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="26" t="inlineStr">
+      <c r="G53" s="12" t="n"/>
+      <c r="H53" s="12" t="n"/>
+      <c r="I53" s="12" t="n"/>
+      <c r="J53" s="12" t="n"/>
+      <c r="K53" s="12" t="n"/>
+      <c r="L53" s="12" t="n"/>
+      <c r="M53" s="12" t="n"/>
+      <c r="N53" s="12" t="n"/>
+      <c r="O53" s="12" t="n"/>
+      <c r="P53" s="12" t="n"/>
+      <c r="Q53" s="12" t="n"/>
+      <c r="R53" s="12" t="n"/>
+      <c r="S53" s="12" t="n"/>
+      <c r="T53" s="12" t="n"/>
+      <c r="U53" s="12" t="n"/>
+      <c r="V53" s="12" t="n"/>
+      <c r="W53" s="12" t="n"/>
+      <c r="X53" s="12" t="n"/>
+      <c r="Y53" s="12" t="n"/>
+      <c r="Z53" s="12" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="26" t="inlineStr">
         <is>
           <t>16:30–17:30</t>
         </is>
       </c>
-      <c r="B53" s="27" t="inlineStr">
+      <c r="B54" s="27" t="inlineStr">
         <is>
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C53" s="44" t="inlineStr">
+      <c r="C54" s="44" t="inlineStr">
         <is>
           <t>Panel 5: The Future of Quantum × AI</t>
         </is>
       </c>
-      <c r="D53" s="44" t="inlineStr">
+      <c r="D54" s="44" t="inlineStr">
         <is>
           <t>Moderator: Philippe Codognet</t>
         </is>
       </c>
-      <c r="E53" s="44" t="inlineStr">
+      <c r="E54" s="44" t="inlineStr">
         <is>
           <t>Shaukat Ali, Simula Research Laboratory; Tadashi Kadowaki, AIST G-QuAT / DENSO; Hoong Chuin Lau, SMU; Jeremy Woo, D-Wave</t>
         </is>
       </c>
-      <c r="F53" s="44" t="n"/>
-      <c r="G53" s="29" t="n"/>
-      <c r="H53" s="29" t="n"/>
-      <c r="I53" s="29" t="n"/>
-      <c r="J53" s="29" t="n"/>
-      <c r="K53" s="29" t="n"/>
-      <c r="L53" s="29" t="n"/>
-      <c r="M53" s="29" t="n"/>
-      <c r="N53" s="29" t="n"/>
-      <c r="O53" s="29" t="n"/>
-      <c r="P53" s="29" t="n"/>
-      <c r="Q53" s="29" t="n"/>
-      <c r="R53" s="29" t="n"/>
-      <c r="S53" s="29" t="n"/>
-      <c r="T53" s="29" t="n"/>
-      <c r="U53" s="29" t="n"/>
-      <c r="V53" s="29" t="n"/>
-      <c r="W53" s="29" t="n"/>
-      <c r="X53" s="29" t="n"/>
-      <c r="Y53" s="29" t="n"/>
-      <c r="Z53" s="29" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="17" t="inlineStr">
+      <c r="F54" s="44" t="n"/>
+      <c r="G54" s="29" t="n"/>
+      <c r="H54" s="29" t="n"/>
+      <c r="I54" s="29" t="n"/>
+      <c r="J54" s="29" t="n"/>
+      <c r="K54" s="29" t="n"/>
+      <c r="L54" s="29" t="n"/>
+      <c r="M54" s="29" t="n"/>
+      <c r="N54" s="29" t="n"/>
+      <c r="O54" s="29" t="n"/>
+      <c r="P54" s="29" t="n"/>
+      <c r="Q54" s="29" t="n"/>
+      <c r="R54" s="29" t="n"/>
+      <c r="S54" s="29" t="n"/>
+      <c r="T54" s="29" t="n"/>
+      <c r="U54" s="29" t="n"/>
+      <c r="V54" s="29" t="n"/>
+      <c r="W54" s="29" t="n"/>
+      <c r="X54" s="29" t="n"/>
+      <c r="Y54" s="29" t="n"/>
+      <c r="Z54" s="29" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="inlineStr">
         <is>
           <t>17:30–18:00</t>
         </is>
       </c>
-      <c r="B54" s="19" t="inlineStr">
+      <c r="B55" s="19" t="inlineStr">
         <is>
           <t>Auditorium 1</t>
         </is>
       </c>
-      <c r="C54" s="58" t="inlineStr">
+      <c r="C55" s="58" t="inlineStr">
         <is>
           <t>Closing Ceremony</t>
-        </is>
-      </c>
-      <c r="D54" s="58" t="n"/>
-      <c r="E54" s="58" t="n"/>
-      <c r="F54" s="58" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="48" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="B55" s="19" t="n"/>
-      <c r="C55" s="58" t="inlineStr">
-        <is>
-          <t>End of Day 3</t>
         </is>
       </c>
       <c r="D55" s="58" t="n"/>
       <c r="E55" s="58" t="n"/>
       <c r="F55" s="58" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="48" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="B56" s="19" t="n"/>
+      <c r="C56" s="58" t="inlineStr">
+        <is>
+          <t>End of Day 3</t>
+        </is>
+      </c>
+      <c r="D56" s="58" t="n"/>
+      <c r="E56" s="58" t="n"/>
+      <c r="F56" s="58" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>